<commit_message>
Add 9 Tips & Tricks samples to readiness checklist (24 samples total)
</commit_message>
<xml_diff>
--- a/doc_readiness_checklist.xlsx
+++ b/doc_readiness_checklist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\AQCWT\OpenCode_Doc\APAI_Chat\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4A50F03D-E2EB-40B0-A0CD-44A9559C5EE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{798329CF-C160-4F7D-B3CE-AD698AE3E867}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{BE8B64C7-7DD3-42E9-8432-DA4C4DC91B80}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="446" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="491" uniqueCount="157">
   <si>
     <t>ID</t>
   </si>
@@ -484,6 +484,33 @@
   </si>
   <si>
     <t>⚠ Documents scoring ≤2 on any criterion need remediation before launch (per Section 5 of AI Testing &amp; Evaluation Plan v1.4)</t>
+  </si>
+  <si>
+    <t>Tips &amp; Tricks – Impose (Folding): Apogee-Impose-Trick_Folding-Direction-Arrow</t>
+  </si>
+  <si>
+    <t>Tips &amp; Tricks – InkDrive: Apogee-InkDrive-Trick_Accurate-CIP3-Presets</t>
+  </si>
+  <si>
+    <t>Tips &amp; Tricks – Proofing: Apogee-Proofing-Trick_GDIProofer-and-Split4ProofApogee</t>
+  </si>
+  <si>
+    <t>Tips &amp; Tricks – Packaging: Apogee-Tips_Apogee-Prepress-with-Packaging-Pack</t>
+  </si>
+  <si>
+    <t>Tips &amp; Tricks – WebApproval: Apogee-Tips_WebApproval-A-Fully-Integrated-Softproof-Solution</t>
+  </si>
+  <si>
+    <t>Tips &amp; Tricks – Automation: Apogee-Trick_Auto-Route-PDF-Files-with-Automate-TP</t>
+  </si>
+  <si>
+    <t>Tips &amp; Tricks – General: The Essential Role of Virus Scanning and Tuning</t>
+  </si>
+  <si>
+    <t>Tips &amp; Tricks – ProductionCenter Dashboard: ProductionCenter-Tips_ECO3-Production-Dashboard</t>
+  </si>
+  <si>
+    <t>Tips &amp; Tricks – ProductionCenter Collaboration: ProductionCenter-Tips_Enhanced-Collaboration</t>
   </si>
 </sst>
 </file>
@@ -621,13 +648,13 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="22" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -3314,10 +3341,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{299327EC-E1E5-4A36-9AAD-A1F4644DF0C0}">
-  <dimension ref="A1:T20"/>
+  <dimension ref="A1:T29"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="67.77734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="80.77734375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="19.77734375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="16.88671875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="7.21875" bestFit="1" customWidth="1"/>
@@ -3340,52 +3367,52 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="17.399999999999999" x14ac:dyDescent="0.35">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="12" t="s">
         <v>116</v>
       </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
-      <c r="F1" s="7"/>
-      <c r="G1" s="7"/>
-      <c r="H1" s="7"/>
-      <c r="I1" s="7"/>
-      <c r="J1" s="7"/>
-      <c r="K1" s="7"/>
-      <c r="L1" s="7"/>
-      <c r="M1" s="7"/>
-      <c r="N1" s="7"/>
-      <c r="O1" s="7"/>
-      <c r="P1" s="7"/>
-      <c r="Q1" s="7"/>
-      <c r="R1" s="7"/>
-      <c r="S1" s="7"/>
-      <c r="T1" s="7"/>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12"/>
+      <c r="H1" s="12"/>
+      <c r="I1" s="12"/>
+      <c r="J1" s="12"/>
+      <c r="K1" s="12"/>
+      <c r="L1" s="12"/>
+      <c r="M1" s="12"/>
+      <c r="N1" s="12"/>
+      <c r="O1" s="12"/>
+      <c r="P1" s="12"/>
+      <c r="Q1" s="12"/>
+      <c r="R1" s="12"/>
+      <c r="S1" s="12"/>
+      <c r="T1" s="12"/>
     </row>
     <row r="2" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A2" s="8" t="s">
+      <c r="A2" s="13" t="s">
         <v>117</v>
       </c>
-      <c r="B2" s="8"/>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="8"/>
-      <c r="F2" s="8"/>
-      <c r="G2" s="8"/>
-      <c r="H2" s="8"/>
-      <c r="I2" s="8"/>
-      <c r="J2" s="8"/>
-      <c r="K2" s="8"/>
-      <c r="L2" s="8"/>
-      <c r="M2" s="8"/>
-      <c r="N2" s="8"/>
-      <c r="O2" s="8"/>
-      <c r="P2" s="8"/>
-      <c r="Q2" s="8"/>
-      <c r="R2" s="8"/>
-      <c r="S2" s="8"/>
-      <c r="T2" s="8"/>
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
+      <c r="F2" s="13"/>
+      <c r="G2" s="13"/>
+      <c r="H2" s="13"/>
+      <c r="I2" s="13"/>
+      <c r="J2" s="13"/>
+      <c r="K2" s="13"/>
+      <c r="L2" s="13"/>
+      <c r="M2" s="13"/>
+      <c r="N2" s="13"/>
+      <c r="O2" s="13"/>
+      <c r="P2" s="13"/>
+      <c r="Q2" s="13"/>
+      <c r="R2" s="13"/>
+      <c r="S2" s="13"/>
+      <c r="T2" s="13"/>
     </row>
     <row r="3" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
@@ -3409,85 +3436,85 @@
       <c r="G3" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="H3" s="9" t="s">
+      <c r="H3" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="I3" s="9" t="s">
+      <c r="I3" s="7" t="s">
         <v>118</v>
       </c>
-      <c r="J3" s="9" t="s">
+      <c r="J3" s="7" t="s">
         <v>119</v>
       </c>
-      <c r="K3" s="10" t="s">
+      <c r="K3" s="8" t="s">
         <v>120</v>
       </c>
-      <c r="L3" s="10" t="s">
+      <c r="L3" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="M3" s="10" t="s">
+      <c r="M3" s="8" t="s">
         <v>122</v>
       </c>
-      <c r="N3" s="10" t="s">
+      <c r="N3" s="8" t="s">
         <v>123</v>
       </c>
-      <c r="O3" s="10" t="s">
+      <c r="O3" s="8" t="s">
         <v>124</v>
       </c>
-      <c r="P3" s="10" t="s">
+      <c r="P3" s="8" t="s">
         <v>125</v>
       </c>
-      <c r="Q3" s="10" t="s">
+      <c r="Q3" s="8" t="s">
         <v>126</v>
       </c>
-      <c r="R3" s="10" t="s">
+      <c r="R3" s="8" t="s">
         <v>127</v>
       </c>
-      <c r="S3" s="10" t="s">
+      <c r="S3" s="8" t="s">
         <v>128</v>
       </c>
-      <c r="T3" s="10" t="s">
+      <c r="T3" s="8" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="4" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A4" s="12" t="s">
+      <c r="A4" s="10" t="s">
         <v>130</v>
       </c>
-      <c r="B4" s="12" t="s">
+      <c r="B4" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="12" t="s">
+      <c r="C4" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="12">
-        <v>14</v>
-      </c>
-      <c r="E4" s="13">
+      <c r="D4" s="10">
+        <v>14</v>
+      </c>
+      <c r="E4" s="11">
         <v>46175.950694444444</v>
       </c>
-      <c r="F4" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="G4" s="12">
+      <c r="F4" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="G4" s="10">
         <v>2</v>
       </c>
-      <c r="H4" s="12">
-        <v>0</v>
-      </c>
-      <c r="I4" s="12"/>
-      <c r="J4" s="12" t="s">
+      <c r="H4" s="10">
+        <v>0</v>
+      </c>
+      <c r="I4" s="10"/>
+      <c r="J4" s="10" t="s">
         <v>131</v>
       </c>
-      <c r="K4" s="11"/>
-      <c r="L4" s="11"/>
-      <c r="M4" s="11"/>
-      <c r="N4" s="11"/>
-      <c r="O4" s="11"/>
-      <c r="P4" s="11"/>
-      <c r="Q4" s="11"/>
-      <c r="R4" s="11"/>
+      <c r="K4" s="9"/>
+      <c r="L4" s="9"/>
+      <c r="M4" s="9"/>
+      <c r="N4" s="9"/>
+      <c r="O4" s="9"/>
+      <c r="P4" s="9"/>
+      <c r="Q4" s="9"/>
+      <c r="R4" s="9"/>
       <c r="S4" t="str">
-        <f>IFERROR(AVERAGE(K4:R4),"")</f>
+        <f t="shared" ref="S4:S18" si="0">IFERROR(AVERAGE(K4:R4),"")</f>
         <v/>
       </c>
     </row>
@@ -3519,58 +3546,58 @@
       <c r="J5" t="s">
         <v>131</v>
       </c>
-      <c r="K5" s="11"/>
-      <c r="L5" s="11"/>
-      <c r="M5" s="11"/>
-      <c r="N5" s="11"/>
-      <c r="O5" s="11"/>
-      <c r="P5" s="11"/>
-      <c r="Q5" s="11"/>
-      <c r="R5" s="11"/>
+      <c r="K5" s="9"/>
+      <c r="L5" s="9"/>
+      <c r="M5" s="9"/>
+      <c r="N5" s="9"/>
+      <c r="O5" s="9"/>
+      <c r="P5" s="9"/>
+      <c r="Q5" s="9"/>
+      <c r="R5" s="9"/>
       <c r="S5" t="str">
-        <f>IFERROR(AVERAGE(K5:R5),"")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
     <row r="6" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A6" s="12" t="s">
+      <c r="A6" s="10" t="s">
         <v>133</v>
       </c>
-      <c r="B6" s="12" t="s">
-        <v>21</v>
-      </c>
-      <c r="C6" s="12" t="s">
+      <c r="B6" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="C6" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="D6" s="12">
-        <v>14</v>
-      </c>
-      <c r="E6" s="13">
+      <c r="D6" s="10">
+        <v>14</v>
+      </c>
+      <c r="E6" s="11">
         <v>46147.351388888892</v>
       </c>
-      <c r="F6" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="G6" s="12">
+      <c r="F6" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="G6" s="10">
         <v>1342</v>
       </c>
-      <c r="H6" s="12">
-        <v>0</v>
-      </c>
-      <c r="I6" s="12"/>
-      <c r="J6" s="12" t="s">
+      <c r="H6" s="10">
+        <v>0</v>
+      </c>
+      <c r="I6" s="10"/>
+      <c r="J6" s="10" t="s">
         <v>131</v>
       </c>
-      <c r="K6" s="11"/>
-      <c r="L6" s="11"/>
-      <c r="M6" s="11"/>
-      <c r="N6" s="11"/>
-      <c r="O6" s="11"/>
-      <c r="P6" s="11"/>
-      <c r="Q6" s="11"/>
-      <c r="R6" s="11"/>
+      <c r="K6" s="9"/>
+      <c r="L6" s="9"/>
+      <c r="M6" s="9"/>
+      <c r="N6" s="9"/>
+      <c r="O6" s="9"/>
+      <c r="P6" s="9"/>
+      <c r="Q6" s="9"/>
+      <c r="R6" s="9"/>
       <c r="S6" t="str">
-        <f>IFERROR(AVERAGE(K6:R6),"")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -3602,58 +3629,58 @@
       <c r="J7" t="s">
         <v>131</v>
       </c>
-      <c r="K7" s="11"/>
-      <c r="L7" s="11"/>
-      <c r="M7" s="11"/>
-      <c r="N7" s="11"/>
-      <c r="O7" s="11"/>
-      <c r="P7" s="11"/>
-      <c r="Q7" s="11"/>
-      <c r="R7" s="11"/>
+      <c r="K7" s="9"/>
+      <c r="L7" s="9"/>
+      <c r="M7" s="9"/>
+      <c r="N7" s="9"/>
+      <c r="O7" s="9"/>
+      <c r="P7" s="9"/>
+      <c r="Q7" s="9"/>
+      <c r="R7" s="9"/>
       <c r="S7" t="str">
-        <f>IFERROR(AVERAGE(K7:R7),"")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
     <row r="8" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A8" s="12" t="s">
+      <c r="A8" s="10" t="s">
         <v>135</v>
       </c>
-      <c r="B8" s="12" t="s">
-        <v>21</v>
-      </c>
-      <c r="C8" s="12" t="s">
+      <c r="B8" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="D8" s="12">
-        <v>14</v>
-      </c>
-      <c r="E8" s="13">
+      <c r="D8" s="10">
+        <v>14</v>
+      </c>
+      <c r="E8" s="11">
         <v>46149.958333333336</v>
       </c>
-      <c r="F8" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="G8" s="12">
+      <c r="F8" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="G8" s="10">
         <v>142</v>
       </c>
-      <c r="H8" s="12">
-        <v>0</v>
-      </c>
-      <c r="I8" s="12"/>
-      <c r="J8" s="12" t="s">
+      <c r="H8" s="10">
+        <v>0</v>
+      </c>
+      <c r="I8" s="10"/>
+      <c r="J8" s="10" t="s">
         <v>131</v>
       </c>
-      <c r="K8" s="11"/>
-      <c r="L8" s="11"/>
-      <c r="M8" s="11"/>
-      <c r="N8" s="11"/>
-      <c r="O8" s="11"/>
-      <c r="P8" s="11"/>
-      <c r="Q8" s="11"/>
-      <c r="R8" s="11"/>
+      <c r="K8" s="9"/>
+      <c r="L8" s="9"/>
+      <c r="M8" s="9"/>
+      <c r="N8" s="9"/>
+      <c r="O8" s="9"/>
+      <c r="P8" s="9"/>
+      <c r="Q8" s="9"/>
+      <c r="R8" s="9"/>
       <c r="S8" t="str">
-        <f>IFERROR(AVERAGE(K8:R8),"")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -3685,58 +3712,58 @@
       <c r="J9" t="s">
         <v>131</v>
       </c>
-      <c r="K9" s="11"/>
-      <c r="L9" s="11"/>
-      <c r="M9" s="11"/>
-      <c r="N9" s="11"/>
-      <c r="O9" s="11"/>
-      <c r="P9" s="11"/>
-      <c r="Q9" s="11"/>
-      <c r="R9" s="11"/>
+      <c r="K9" s="9"/>
+      <c r="L9" s="9"/>
+      <c r="M9" s="9"/>
+      <c r="N9" s="9"/>
+      <c r="O9" s="9"/>
+      <c r="P9" s="9"/>
+      <c r="Q9" s="9"/>
+      <c r="R9" s="9"/>
       <c r="S9" t="str">
-        <f>IFERROR(AVERAGE(K9:R9),"")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
     <row r="10" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A10" s="12" t="s">
+      <c r="A10" s="10" t="s">
         <v>137</v>
       </c>
-      <c r="B10" s="12" t="s">
-        <v>21</v>
-      </c>
-      <c r="C10" s="12" t="s">
-        <v>49</v>
-      </c>
-      <c r="D10" s="12">
-        <v>14</v>
-      </c>
-      <c r="E10" s="13">
+      <c r="B10" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="C10" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="D10" s="10">
+        <v>14</v>
+      </c>
+      <c r="E10" s="11">
         <v>46162.013194444444</v>
       </c>
-      <c r="F10" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="G10" s="12">
+      <c r="F10" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="G10" s="10">
         <v>12</v>
       </c>
-      <c r="H10" s="12">
-        <v>0</v>
-      </c>
-      <c r="I10" s="12"/>
-      <c r="J10" s="12" t="s">
+      <c r="H10" s="10">
+        <v>0</v>
+      </c>
+      <c r="I10" s="10"/>
+      <c r="J10" s="10" t="s">
         <v>131</v>
       </c>
-      <c r="K10" s="11"/>
-      <c r="L10" s="11"/>
-      <c r="M10" s="11"/>
-      <c r="N10" s="11"/>
-      <c r="O10" s="11"/>
-      <c r="P10" s="11"/>
-      <c r="Q10" s="11"/>
-      <c r="R10" s="11"/>
+      <c r="K10" s="9"/>
+      <c r="L10" s="9"/>
+      <c r="M10" s="9"/>
+      <c r="N10" s="9"/>
+      <c r="O10" s="9"/>
+      <c r="P10" s="9"/>
+      <c r="Q10" s="9"/>
+      <c r="R10" s="9"/>
       <c r="S10" t="str">
-        <f>IFERROR(AVERAGE(K10:R10),"")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -3768,58 +3795,58 @@
       <c r="J11" t="s">
         <v>131</v>
       </c>
-      <c r="K11" s="11"/>
-      <c r="L11" s="11"/>
-      <c r="M11" s="11"/>
-      <c r="N11" s="11"/>
-      <c r="O11" s="11"/>
-      <c r="P11" s="11"/>
-      <c r="Q11" s="11"/>
-      <c r="R11" s="11"/>
+      <c r="K11" s="9"/>
+      <c r="L11" s="9"/>
+      <c r="M11" s="9"/>
+      <c r="N11" s="9"/>
+      <c r="O11" s="9"/>
+      <c r="P11" s="9"/>
+      <c r="Q11" s="9"/>
+      <c r="R11" s="9"/>
       <c r="S11" t="str">
-        <f>IFERROR(AVERAGE(K11:R11),"")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
     <row r="12" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A12" s="12" t="s">
+      <c r="A12" s="10" t="s">
         <v>139</v>
       </c>
-      <c r="B12" s="12" t="s">
-        <v>21</v>
-      </c>
-      <c r="C12" s="12" t="s">
-        <v>49</v>
-      </c>
-      <c r="D12" s="12">
-        <v>14</v>
-      </c>
-      <c r="E12" s="13">
+      <c r="B12" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="C12" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="D12" s="10">
+        <v>14</v>
+      </c>
+      <c r="E12" s="11">
         <v>46149.957638888889</v>
       </c>
-      <c r="F12" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="G12" s="12">
+      <c r="F12" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="G12" s="10">
         <v>16</v>
       </c>
-      <c r="H12" s="12">
-        <v>0</v>
-      </c>
-      <c r="I12" s="12"/>
-      <c r="J12" s="12" t="s">
+      <c r="H12" s="10">
+        <v>0</v>
+      </c>
+      <c r="I12" s="10"/>
+      <c r="J12" s="10" t="s">
         <v>131</v>
       </c>
-      <c r="K12" s="11"/>
-      <c r="L12" s="11"/>
-      <c r="M12" s="11"/>
-      <c r="N12" s="11"/>
-      <c r="O12" s="11"/>
-      <c r="P12" s="11"/>
-      <c r="Q12" s="11"/>
-      <c r="R12" s="11"/>
+      <c r="K12" s="9"/>
+      <c r="L12" s="9"/>
+      <c r="M12" s="9"/>
+      <c r="N12" s="9"/>
+      <c r="O12" s="9"/>
+      <c r="P12" s="9"/>
+      <c r="Q12" s="9"/>
+      <c r="R12" s="9"/>
       <c r="S12" t="str">
-        <f>IFERROR(AVERAGE(K12:R12),"")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -3851,58 +3878,58 @@
       <c r="J13" t="s">
         <v>131</v>
       </c>
-      <c r="K13" s="11"/>
-      <c r="L13" s="11"/>
-      <c r="M13" s="11"/>
-      <c r="N13" s="11"/>
-      <c r="O13" s="11"/>
-      <c r="P13" s="11"/>
-      <c r="Q13" s="11"/>
-      <c r="R13" s="11"/>
+      <c r="K13" s="9"/>
+      <c r="L13" s="9"/>
+      <c r="M13" s="9"/>
+      <c r="N13" s="9"/>
+      <c r="O13" s="9"/>
+      <c r="P13" s="9"/>
+      <c r="Q13" s="9"/>
+      <c r="R13" s="9"/>
       <c r="S13" t="str">
-        <f>IFERROR(AVERAGE(K13:R13),"")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
     <row r="14" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A14" s="12" t="s">
+      <c r="A14" s="10" t="s">
         <v>141</v>
       </c>
-      <c r="B14" s="12" t="s">
-        <v>21</v>
-      </c>
-      <c r="C14" s="12" t="s">
-        <v>49</v>
-      </c>
-      <c r="D14" s="12">
+      <c r="B14" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="C14" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="D14" s="10">
         <v>15</v>
       </c>
-      <c r="E14" s="13">
+      <c r="E14" s="11">
         <v>46162.022916666669</v>
       </c>
-      <c r="F14" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="G14" s="12">
-        <v>21</v>
-      </c>
-      <c r="H14" s="12">
-        <v>0</v>
-      </c>
-      <c r="I14" s="12"/>
-      <c r="J14" s="12" t="s">
+      <c r="F14" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="G14" s="10">
+        <v>21</v>
+      </c>
+      <c r="H14" s="10">
+        <v>0</v>
+      </c>
+      <c r="I14" s="10"/>
+      <c r="J14" s="10" t="s">
         <v>131</v>
       </c>
-      <c r="K14" s="11"/>
-      <c r="L14" s="11"/>
-      <c r="M14" s="11"/>
-      <c r="N14" s="11"/>
-      <c r="O14" s="11"/>
-      <c r="P14" s="11"/>
-      <c r="Q14" s="11"/>
-      <c r="R14" s="11"/>
+      <c r="K14" s="9"/>
+      <c r="L14" s="9"/>
+      <c r="M14" s="9"/>
+      <c r="N14" s="9"/>
+      <c r="O14" s="9"/>
+      <c r="P14" s="9"/>
+      <c r="Q14" s="9"/>
+      <c r="R14" s="9"/>
       <c r="S14" t="str">
-        <f>IFERROR(AVERAGE(K14:R14),"")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -3934,60 +3961,60 @@
       <c r="J15" t="s">
         <v>131</v>
       </c>
-      <c r="K15" s="11"/>
-      <c r="L15" s="11"/>
-      <c r="M15" s="11"/>
-      <c r="N15" s="11"/>
-      <c r="O15" s="11"/>
-      <c r="P15" s="11"/>
-      <c r="Q15" s="11"/>
-      <c r="R15" s="11"/>
+      <c r="K15" s="9"/>
+      <c r="L15" s="9"/>
+      <c r="M15" s="9"/>
+      <c r="N15" s="9"/>
+      <c r="O15" s="9"/>
+      <c r="P15" s="9"/>
+      <c r="Q15" s="9"/>
+      <c r="R15" s="9"/>
       <c r="S15" t="str">
-        <f>IFERROR(AVERAGE(K15:R15),"")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
     <row r="16" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A16" s="12" t="s">
+      <c r="A16" s="10" t="s">
         <v>143</v>
       </c>
-      <c r="B16" s="12" t="s">
+      <c r="B16" s="10" t="s">
         <v>101</v>
       </c>
-      <c r="C16" s="12" t="s">
+      <c r="C16" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="D16" s="12">
-        <v>14</v>
-      </c>
-      <c r="E16" s="13">
+      <c r="D16" s="10">
+        <v>14</v>
+      </c>
+      <c r="E16" s="11">
         <v>46147.338888888888</v>
       </c>
-      <c r="F16" s="12" t="s">
+      <c r="F16" s="10" t="s">
         <v>95</v>
       </c>
-      <c r="G16" s="12">
+      <c r="G16" s="10">
         <v>278</v>
       </c>
-      <c r="H16" s="12">
-        <v>0</v>
-      </c>
-      <c r="I16" s="12" t="s">
+      <c r="H16" s="10">
+        <v>0</v>
+      </c>
+      <c r="I16" s="10" t="s">
         <v>144</v>
       </c>
-      <c r="J16" s="12" t="s">
+      <c r="J16" s="10" t="s">
         <v>131</v>
       </c>
-      <c r="K16" s="11"/>
-      <c r="L16" s="11"/>
-      <c r="M16" s="11"/>
-      <c r="N16" s="11"/>
-      <c r="O16" s="11"/>
-      <c r="P16" s="11"/>
-      <c r="Q16" s="11"/>
-      <c r="R16" s="11"/>
+      <c r="K16" s="9"/>
+      <c r="L16" s="9"/>
+      <c r="M16" s="9"/>
+      <c r="N16" s="9"/>
+      <c r="O16" s="9"/>
+      <c r="P16" s="9"/>
+      <c r="Q16" s="9"/>
+      <c r="R16" s="9"/>
       <c r="S16" t="str">
-        <f>IFERROR(AVERAGE(K16:R16),"")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -4019,92 +4046,466 @@
       <c r="J17" t="s">
         <v>131</v>
       </c>
-      <c r="K17" s="11"/>
-      <c r="L17" s="11"/>
-      <c r="M17" s="11"/>
-      <c r="N17" s="11"/>
-      <c r="O17" s="11"/>
-      <c r="P17" s="11"/>
-      <c r="Q17" s="11"/>
-      <c r="R17" s="11"/>
+      <c r="K17" s="9"/>
+      <c r="L17" s="9"/>
+      <c r="M17" s="9"/>
+      <c r="N17" s="9"/>
+      <c r="O17" s="9"/>
+      <c r="P17" s="9"/>
+      <c r="Q17" s="9"/>
+      <c r="R17" s="9"/>
       <c r="S17" t="str">
-        <f>IFERROR(AVERAGE(K17:R17),"")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
     <row r="18" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A18" s="12" t="s">
+      <c r="A18" s="10" t="s">
         <v>146</v>
       </c>
-      <c r="B18" s="12" t="s">
+      <c r="B18" s="10" t="s">
         <v>101</v>
       </c>
-      <c r="C18" s="12" t="s">
-        <v>49</v>
-      </c>
-      <c r="D18" s="12">
-        <v>14</v>
-      </c>
-      <c r="E18" s="13">
+      <c r="C18" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="D18" s="10">
+        <v>14</v>
+      </c>
+      <c r="E18" s="11">
         <v>46162.020833333336</v>
       </c>
-      <c r="F18" s="12" t="s">
+      <c r="F18" s="10" t="s">
         <v>95</v>
       </c>
-      <c r="G18" s="12">
+      <c r="G18" s="10">
         <v>15</v>
       </c>
-      <c r="H18" s="12">
-        <v>0</v>
-      </c>
-      <c r="I18" s="12" t="s">
+      <c r="H18" s="10">
+        <v>0</v>
+      </c>
+      <c r="I18" s="10" t="s">
         <v>144</v>
       </c>
-      <c r="J18" s="12" t="s">
+      <c r="J18" s="10" t="s">
         <v>131</v>
       </c>
-      <c r="K18" s="11"/>
-      <c r="L18" s="11"/>
-      <c r="M18" s="11"/>
-      <c r="N18" s="11"/>
-      <c r="O18" s="11"/>
-      <c r="P18" s="11"/>
-      <c r="Q18" s="11"/>
-      <c r="R18" s="11"/>
+      <c r="K18" s="9"/>
+      <c r="L18" s="9"/>
+      <c r="M18" s="9"/>
+      <c r="N18" s="9"/>
+      <c r="O18" s="9"/>
+      <c r="P18" s="9"/>
+      <c r="Q18" s="9"/>
+      <c r="R18" s="9"/>
       <c r="S18" t="str">
-        <f>IFERROR(AVERAGE(K18:R18),"")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
     <row r="20" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A20" s="14" t="s">
+      <c r="A20" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="B20" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="C20" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="D20" s="10">
+        <v>14</v>
+      </c>
+      <c r="E20" s="11">
+        <v>46175.950694444444</v>
+      </c>
+      <c r="F20" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="G20" s="10">
+        <v>1</v>
+      </c>
+      <c r="H20" s="10">
+        <v>0</v>
+      </c>
+      <c r="I20" s="10"/>
+      <c r="J20" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="K20" s="9"/>
+      <c r="L20" s="9"/>
+      <c r="M20" s="9"/>
+      <c r="N20" s="9"/>
+      <c r="O20" s="9"/>
+      <c r="P20" s="9"/>
+      <c r="Q20" s="9"/>
+      <c r="R20" s="9"/>
+      <c r="S20" t="str">
+        <f>IFERROR(AVERAGE(K20:R20),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>149</v>
+      </c>
+      <c r="B21" t="s">
+        <v>11</v>
+      </c>
+      <c r="C21" t="s">
+        <v>12</v>
+      </c>
+      <c r="D21">
+        <v>14</v>
+      </c>
+      <c r="E21" s="2">
+        <v>46175.950694444444</v>
+      </c>
+      <c r="F21" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G21">
+        <v>2</v>
+      </c>
+      <c r="H21">
+        <v>0</v>
+      </c>
+      <c r="J21" t="s">
+        <v>131</v>
+      </c>
+      <c r="K21" s="9"/>
+      <c r="L21" s="9"/>
+      <c r="M21" s="9"/>
+      <c r="N21" s="9"/>
+      <c r="O21" s="9"/>
+      <c r="P21" s="9"/>
+      <c r="Q21" s="9"/>
+      <c r="R21" s="9"/>
+      <c r="S21" t="str">
+        <f>IFERROR(AVERAGE(K21:R21),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A22" s="10" t="s">
+        <v>150</v>
+      </c>
+      <c r="B22" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="C22" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="D22" s="10">
+        <v>14</v>
+      </c>
+      <c r="E22" s="11">
+        <v>46161.998611111114</v>
+      </c>
+      <c r="F22" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="G22" s="10">
+        <v>1</v>
+      </c>
+      <c r="H22" s="10">
+        <v>0</v>
+      </c>
+      <c r="I22" s="10"/>
+      <c r="J22" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="K22" s="9"/>
+      <c r="L22" s="9"/>
+      <c r="M22" s="9"/>
+      <c r="N22" s="9"/>
+      <c r="O22" s="9"/>
+      <c r="P22" s="9"/>
+      <c r="Q22" s="9"/>
+      <c r="R22" s="9"/>
+      <c r="S22" t="str">
+        <f>IFERROR(AVERAGE(K22:R22),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>151</v>
+      </c>
+      <c r="B23" t="s">
+        <v>21</v>
+      </c>
+      <c r="C23" t="s">
+        <v>19</v>
+      </c>
+      <c r="D23">
+        <v>14</v>
+      </c>
+      <c r="E23" s="2">
+        <v>46161.998611111114</v>
+      </c>
+      <c r="F23" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G23">
+        <v>3</v>
+      </c>
+      <c r="H23">
+        <v>0</v>
+      </c>
+      <c r="J23" t="s">
+        <v>131</v>
+      </c>
+      <c r="K23" s="9"/>
+      <c r="L23" s="9"/>
+      <c r="M23" s="9"/>
+      <c r="N23" s="9"/>
+      <c r="O23" s="9"/>
+      <c r="P23" s="9"/>
+      <c r="Q23" s="9"/>
+      <c r="R23" s="9"/>
+      <c r="S23" t="str">
+        <f>IFERROR(AVERAGE(K23:R23),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A24" s="10" t="s">
+        <v>152</v>
+      </c>
+      <c r="B24" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="C24" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="D24" s="10">
+        <v>14</v>
+      </c>
+      <c r="E24" s="11">
+        <v>46161.998611111114</v>
+      </c>
+      <c r="F24" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="G24" s="10">
+        <v>10</v>
+      </c>
+      <c r="H24" s="10">
+        <v>0</v>
+      </c>
+      <c r="I24" s="10"/>
+      <c r="J24" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="K24" s="9"/>
+      <c r="L24" s="9"/>
+      <c r="M24" s="9"/>
+      <c r="N24" s="9"/>
+      <c r="O24" s="9"/>
+      <c r="P24" s="9"/>
+      <c r="Q24" s="9"/>
+      <c r="R24" s="9"/>
+      <c r="S24" t="str">
+        <f>IFERROR(AVERAGE(K24:R24),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>153</v>
+      </c>
+      <c r="B25" t="s">
+        <v>21</v>
+      </c>
+      <c r="C25" t="s">
+        <v>19</v>
+      </c>
+      <c r="D25">
+        <v>14</v>
+      </c>
+      <c r="E25" s="2">
+        <v>46161.998611111114</v>
+      </c>
+      <c r="F25" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G25">
+        <v>2</v>
+      </c>
+      <c r="H25">
+        <v>0</v>
+      </c>
+      <c r="J25" t="s">
+        <v>131</v>
+      </c>
+      <c r="K25" s="9"/>
+      <c r="L25" s="9"/>
+      <c r="M25" s="9"/>
+      <c r="N25" s="9"/>
+      <c r="O25" s="9"/>
+      <c r="P25" s="9"/>
+      <c r="Q25" s="9"/>
+      <c r="R25" s="9"/>
+      <c r="S25" t="str">
+        <f>IFERROR(AVERAGE(K25:R25),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A26" s="10" t="s">
+        <v>154</v>
+      </c>
+      <c r="B26" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="C26" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="D26" s="10">
+        <v>14</v>
+      </c>
+      <c r="E26" s="11">
+        <v>46161.998611111114</v>
+      </c>
+      <c r="F26" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="G26" s="10">
+        <v>1</v>
+      </c>
+      <c r="H26" s="10">
+        <v>0</v>
+      </c>
+      <c r="I26" s="10"/>
+      <c r="J26" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="K26" s="9"/>
+      <c r="L26" s="9"/>
+      <c r="M26" s="9"/>
+      <c r="N26" s="9"/>
+      <c r="O26" s="9"/>
+      <c r="P26" s="9"/>
+      <c r="Q26" s="9"/>
+      <c r="R26" s="9"/>
+      <c r="S26" t="str">
+        <f>IFERROR(AVERAGE(K26:R26),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>155</v>
+      </c>
+      <c r="B27" t="s">
+        <v>101</v>
+      </c>
+      <c r="C27" t="s">
+        <v>19</v>
+      </c>
+      <c r="D27">
+        <v>14</v>
+      </c>
+      <c r="E27" s="2">
+        <v>46161.992361111108</v>
+      </c>
+      <c r="F27" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G27">
+        <v>3</v>
+      </c>
+      <c r="H27">
+        <v>0</v>
+      </c>
+      <c r="J27" t="s">
+        <v>131</v>
+      </c>
+      <c r="K27" s="9"/>
+      <c r="L27" s="9"/>
+      <c r="M27" s="9"/>
+      <c r="N27" s="9"/>
+      <c r="O27" s="9"/>
+      <c r="P27" s="9"/>
+      <c r="Q27" s="9"/>
+      <c r="R27" s="9"/>
+      <c r="S27" t="str">
+        <f>IFERROR(AVERAGE(K27:R27),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A28" s="10" t="s">
+        <v>156</v>
+      </c>
+      <c r="B28" s="10" t="s">
+        <v>101</v>
+      </c>
+      <c r="C28" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="D28" s="10">
+        <v>14</v>
+      </c>
+      <c r="E28" s="11">
+        <v>46161.993750000001</v>
+      </c>
+      <c r="F28" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="G28" s="10">
+        <v>9</v>
+      </c>
+      <c r="H28" s="10">
+        <v>0</v>
+      </c>
+      <c r="I28" s="10"/>
+      <c r="J28" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="K28" s="9"/>
+      <c r="L28" s="9"/>
+      <c r="M28" s="9"/>
+      <c r="N28" s="9"/>
+      <c r="O28" s="9"/>
+      <c r="P28" s="9"/>
+      <c r="Q28" s="9"/>
+      <c r="R28" s="9"/>
+      <c r="S28" t="str">
+        <f>IFERROR(AVERAGE(K28:R28),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A29" s="14" t="s">
         <v>147</v>
       </c>
-      <c r="B20" s="14"/>
-      <c r="C20" s="14"/>
-      <c r="D20" s="14"/>
-      <c r="E20" s="14"/>
-      <c r="F20" s="14"/>
-      <c r="G20" s="14"/>
-      <c r="H20" s="14"/>
-      <c r="I20" s="14"/>
-      <c r="J20" s="14"/>
-      <c r="K20" s="14"/>
-      <c r="L20" s="14"/>
-      <c r="M20" s="14"/>
-      <c r="N20" s="14"/>
-      <c r="O20" s="14"/>
-      <c r="P20" s="14"/>
-      <c r="Q20" s="14"/>
-      <c r="R20" s="14"/>
-      <c r="S20" s="14"/>
-      <c r="T20" s="14"/>
+      <c r="B29" s="14"/>
+      <c r="C29" s="14"/>
+      <c r="D29" s="14"/>
+      <c r="E29" s="14"/>
+      <c r="F29" s="14"/>
+      <c r="G29" s="14"/>
+      <c r="H29" s="14"/>
+      <c r="I29" s="14"/>
+      <c r="J29" s="14"/>
+      <c r="K29" s="14"/>
+      <c r="L29" s="14"/>
+      <c r="M29" s="14"/>
+      <c r="N29" s="14"/>
+      <c r="O29" s="14"/>
+      <c r="P29" s="14"/>
+      <c r="Q29" s="14"/>
+      <c r="R29" s="14"/>
+      <c r="S29" s="14"/>
+      <c r="T29" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:T1"/>
     <mergeCell ref="A2:T2"/>
-    <mergeCell ref="A20:T20"/>
+    <mergeCell ref="A29:T29"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Score readiness checklist for 3 sample docs (rows 4, 20, 21)
</commit_message>
<xml_diff>
--- a/doc_readiness_checklist.xlsx
+++ b/doc_readiness_checklist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\AQCWT\OpenCode_Doc\APAI_Chat\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{798329CF-C160-4F7D-B3CE-AD698AE3E867}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{896CCC29-AD64-4393-B000-1A9F1077B684}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{BE8B64C7-7DD3-42E9-8432-DA4C4DC91B80}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="491" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="492" uniqueCount="158">
   <si>
     <t>ID</t>
   </si>
@@ -511,6 +511,9 @@
   </si>
   <si>
     <t>Tips &amp; Tricks – ProductionCenter Collaboration: ProductionCenter-Tips_Enhanced-Collaboration</t>
+  </si>
+  <si>
+    <t>Criterion 5 (Text/Image Ratio=2): Key fold direction information relies heavily on images; add text description of arrow direction.</t>
   </si>
 </sst>
 </file>
@@ -3505,17 +3508,33 @@
       <c r="J4" s="10" t="s">
         <v>131</v>
       </c>
-      <c r="K4" s="9"/>
-      <c r="L4" s="9"/>
-      <c r="M4" s="9"/>
-      <c r="N4" s="9"/>
-      <c r="O4" s="9"/>
-      <c r="P4" s="9"/>
-      <c r="Q4" s="9"/>
-      <c r="R4" s="9"/>
-      <c r="S4" t="str">
+      <c r="K4" s="9">
+        <v>4</v>
+      </c>
+      <c r="L4" s="9">
+        <v>4</v>
+      </c>
+      <c r="M4" s="9">
+        <v>4</v>
+      </c>
+      <c r="N4" s="9">
+        <v>4</v>
+      </c>
+      <c r="O4" s="9">
+        <v>3</v>
+      </c>
+      <c r="P4" s="9">
+        <v>4</v>
+      </c>
+      <c r="Q4" s="9">
+        <v>3</v>
+      </c>
+      <c r="R4" s="9">
+        <v>4</v>
+      </c>
+      <c r="S4">
         <f t="shared" ref="S4:S18" si="0">IFERROR(AVERAGE(K4:R4),"")</f>
-        <v/>
+        <v>3.75</v>
       </c>
     </row>
     <row r="5" spans="1:20" x14ac:dyDescent="0.3">
@@ -4132,17 +4151,36 @@
       <c r="J20" s="10" t="s">
         <v>131</v>
       </c>
-      <c r="K20" s="9"/>
-      <c r="L20" s="9"/>
-      <c r="M20" s="9"/>
-      <c r="N20" s="9"/>
-      <c r="O20" s="9"/>
-      <c r="P20" s="9"/>
-      <c r="Q20" s="9"/>
-      <c r="R20" s="9"/>
-      <c r="S20" t="str">
-        <f>IFERROR(AVERAGE(K20:R20),"")</f>
-        <v/>
+      <c r="K20" s="9">
+        <v>3</v>
+      </c>
+      <c r="L20" s="9">
+        <v>4</v>
+      </c>
+      <c r="M20" s="9">
+        <v>4</v>
+      </c>
+      <c r="N20" s="9">
+        <v>4</v>
+      </c>
+      <c r="O20" s="9">
+        <v>2</v>
+      </c>
+      <c r="P20" s="9">
+        <v>3</v>
+      </c>
+      <c r="Q20" s="9">
+        <v>3</v>
+      </c>
+      <c r="R20" s="9">
+        <v>4</v>
+      </c>
+      <c r="S20">
+        <f t="shared" ref="S20:S28" si="1">IFERROR(AVERAGE(K20:R20),"")</f>
+        <v>3.375</v>
+      </c>
+      <c r="T20" t="s">
+        <v>157</v>
       </c>
     </row>
     <row r="21" spans="1:20" x14ac:dyDescent="0.3">
@@ -4173,17 +4211,33 @@
       <c r="J21" t="s">
         <v>131</v>
       </c>
-      <c r="K21" s="9"/>
-      <c r="L21" s="9"/>
-      <c r="M21" s="9"/>
-      <c r="N21" s="9"/>
-      <c r="O21" s="9"/>
-      <c r="P21" s="9"/>
-      <c r="Q21" s="9"/>
-      <c r="R21" s="9"/>
-      <c r="S21" t="str">
-        <f>IFERROR(AVERAGE(K21:R21),"")</f>
-        <v/>
+      <c r="K21" s="9">
+        <v>3</v>
+      </c>
+      <c r="L21" s="9">
+        <v>4</v>
+      </c>
+      <c r="M21" s="9">
+        <v>4</v>
+      </c>
+      <c r="N21" s="9">
+        <v>4</v>
+      </c>
+      <c r="O21" s="9">
+        <v>3</v>
+      </c>
+      <c r="P21" s="9">
+        <v>3</v>
+      </c>
+      <c r="Q21" s="9">
+        <v>3</v>
+      </c>
+      <c r="R21" s="9">
+        <v>4</v>
+      </c>
+      <c r="S21">
+        <f t="shared" si="1"/>
+        <v>3.5</v>
       </c>
     </row>
     <row r="22" spans="1:20" x14ac:dyDescent="0.3">
@@ -4224,7 +4278,7 @@
       <c r="Q22" s="9"/>
       <c r="R22" s="9"/>
       <c r="S22" t="str">
-        <f>IFERROR(AVERAGE(K22:R22),"")</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
@@ -4265,7 +4319,7 @@
       <c r="Q23" s="9"/>
       <c r="R23" s="9"/>
       <c r="S23" t="str">
-        <f>IFERROR(AVERAGE(K23:R23),"")</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
@@ -4307,7 +4361,7 @@
       <c r="Q24" s="9"/>
       <c r="R24" s="9"/>
       <c r="S24" t="str">
-        <f>IFERROR(AVERAGE(K24:R24),"")</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
@@ -4348,7 +4402,7 @@
       <c r="Q25" s="9"/>
       <c r="R25" s="9"/>
       <c r="S25" t="str">
-        <f>IFERROR(AVERAGE(K25:R25),"")</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
@@ -4390,7 +4444,7 @@
       <c r="Q26" s="9"/>
       <c r="R26" s="9"/>
       <c r="S26" t="str">
-        <f>IFERROR(AVERAGE(K26:R26),"")</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
@@ -4431,7 +4485,7 @@
       <c r="Q27" s="9"/>
       <c r="R27" s="9"/>
       <c r="S27" t="str">
-        <f>IFERROR(AVERAGE(K27:R27),"")</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
@@ -4473,7 +4527,7 @@
       <c r="Q28" s="9"/>
       <c r="R28" s="9"/>
       <c r="S28" t="str">
-        <f>IFERROR(AVERAGE(K28:R28),"")</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Update checklist: add readiness scores for ProductionCenter_UG_14.0_en-US (row 16, avg 4.00)
</commit_message>
<xml_diff>
--- a/doc_readiness_checklist.xlsx
+++ b/doc_readiness_checklist.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\AQCWT\OpenCode_Doc\APAI_Chat\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{896CCC29-AD64-4393-B000-1A9F1077B684}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B824B558-9DA6-4130-9CB3-E654E095EA33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{BE8B64C7-7DD3-42E9-8432-DA4C4DC91B80}"/>
+    <workbookView xWindow="5364" yWindow="1572" windowWidth="13836" windowHeight="7116" activeTab="1" xr2:uid="{BE8B64C7-7DD3-42E9-8432-DA4C4DC91B80}"/>
   </bookViews>
   <sheets>
     <sheet name="All Documents – Status" sheetId="1" r:id="rId1"/>
@@ -4024,17 +4024,33 @@
       <c r="J16" s="10" t="s">
         <v>131</v>
       </c>
-      <c r="K16" s="9"/>
-      <c r="L16" s="9"/>
-      <c r="M16" s="9"/>
-      <c r="N16" s="9"/>
-      <c r="O16" s="9"/>
-      <c r="P16" s="9"/>
-      <c r="Q16" s="9"/>
-      <c r="R16" s="9"/>
-      <c r="S16" t="str">
+      <c r="K16" s="9">
+        <v>5</v>
+      </c>
+      <c r="L16" s="9">
+        <v>3</v>
+      </c>
+      <c r="M16" s="9">
+        <v>4</v>
+      </c>
+      <c r="N16" s="9">
+        <v>5</v>
+      </c>
+      <c r="O16" s="9">
+        <v>4</v>
+      </c>
+      <c r="P16" s="9">
+        <v>5</v>
+      </c>
+      <c r="Q16" s="9">
+        <v>3</v>
+      </c>
+      <c r="R16" s="9">
+        <v>3</v>
+      </c>
+      <c r="S16">
         <f t="shared" si="0"/>
-        <v/>
+        <v>4</v>
       </c>
     </row>
     <row r="17" spans="1:20" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Task 2: score 10 more documents (batch 2) — 14 of 24 complete
</commit_message>
<xml_diff>
--- a/doc_readiness_checklist.xlsx
+++ b/doc_readiness_checklist.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\AQCWT\OpenCode_Doc\APAI_Chat\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B824B558-9DA6-4130-9CB3-E654E095EA33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CF5B6D5-D258-4560-9532-A0D71112C962}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5364" yWindow="1572" windowWidth="13836" windowHeight="7116" activeTab="1" xr2:uid="{BE8B64C7-7DD3-42E9-8432-DA4C4DC91B80}"/>
+    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{BE8B64C7-7DD3-42E9-8432-DA4C4DC91B80}"/>
   </bookViews>
   <sheets>
     <sheet name="All Documents – Status" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="492" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="498" uniqueCount="164">
   <si>
     <t>ID</t>
   </si>
@@ -514,6 +514,24 @@
   </si>
   <si>
     <t>Criterion 5 (Text/Image Ratio=2): Key fold direction information relies heavily on images; add text description of arrow direction.</t>
+  </si>
+  <si>
+    <t>C7=2: No troubleshooting content for annotation or notification failures.</t>
+  </si>
+  <si>
+    <t>C7=2: No troubleshooting content for data access or dashboard issues.</t>
+  </si>
+  <si>
+    <t>C6=2: Overview only; links to external tutorials but no procedural steps in document. C7=2: No troubleshooting content.</t>
+  </si>
+  <si>
+    <t>C6=2: No procedure steps for DQS activation or configuration. C7=2: No troubleshooting content.</t>
+  </si>
+  <si>
+    <t>C1=2: No internal section headings within body text. C6=2: Feature description only - no setup or usage steps included. C7=2: No error or troubleshooting content.</t>
+  </si>
+  <si>
+    <t>C7=2: No troubleshooting scenarios for passkey failures or browser compatibility issues.</t>
   </si>
 </sst>
 </file>
@@ -3565,17 +3583,36 @@
       <c r="J5" t="s">
         <v>131</v>
       </c>
-      <c r="K5" s="9"/>
-      <c r="L5" s="9"/>
-      <c r="M5" s="9"/>
-      <c r="N5" s="9"/>
-      <c r="O5" s="9"/>
-      <c r="P5" s="9"/>
-      <c r="Q5" s="9"/>
-      <c r="R5" s="9"/>
-      <c r="S5" t="str">
+      <c r="K5" s="9">
+        <v>3</v>
+      </c>
+      <c r="L5" s="9">
+        <v>4</v>
+      </c>
+      <c r="M5" s="9">
+        <v>4</v>
+      </c>
+      <c r="N5" s="9">
+        <v>4</v>
+      </c>
+      <c r="O5" s="9">
+        <v>5</v>
+      </c>
+      <c r="P5" s="9">
+        <v>2</v>
+      </c>
+      <c r="Q5" s="9">
+        <v>2</v>
+      </c>
+      <c r="R5" s="9">
+        <v>4</v>
+      </c>
+      <c r="S5">
         <f t="shared" si="0"/>
-        <v/>
+        <v>3.5</v>
+      </c>
+      <c r="T5" t="s">
+        <v>161</v>
       </c>
     </row>
     <row r="6" spans="1:20" x14ac:dyDescent="0.3">
@@ -3773,17 +3810,33 @@
       <c r="J10" s="10" t="s">
         <v>131</v>
       </c>
-      <c r="K10" s="9"/>
-      <c r="L10" s="9"/>
-      <c r="M10" s="9"/>
-      <c r="N10" s="9"/>
-      <c r="O10" s="9"/>
-      <c r="P10" s="9"/>
-      <c r="Q10" s="9"/>
-      <c r="R10" s="9"/>
-      <c r="S10" t="str">
+      <c r="K10" s="9">
+        <v>4</v>
+      </c>
+      <c r="L10" s="9">
+        <v>3</v>
+      </c>
+      <c r="M10" s="9">
+        <v>4</v>
+      </c>
+      <c r="N10" s="9">
+        <v>5</v>
+      </c>
+      <c r="O10" s="9">
+        <v>3</v>
+      </c>
+      <c r="P10" s="9">
+        <v>5</v>
+      </c>
+      <c r="Q10" s="9">
+        <v>3</v>
+      </c>
+      <c r="R10" s="9">
+        <v>3</v>
+      </c>
+      <c r="S10">
         <f t="shared" si="0"/>
-        <v/>
+        <v>3.75</v>
       </c>
     </row>
     <row r="11" spans="1:20" x14ac:dyDescent="0.3">
@@ -4081,17 +4134,36 @@
       <c r="J17" t="s">
         <v>131</v>
       </c>
-      <c r="K17" s="9"/>
-      <c r="L17" s="9"/>
-      <c r="M17" s="9"/>
-      <c r="N17" s="9"/>
-      <c r="O17" s="9"/>
-      <c r="P17" s="9"/>
-      <c r="Q17" s="9"/>
-      <c r="R17" s="9"/>
-      <c r="S17" t="str">
+      <c r="K17" s="9">
+        <v>3</v>
+      </c>
+      <c r="L17" s="9">
+        <v>4</v>
+      </c>
+      <c r="M17" s="9">
+        <v>4</v>
+      </c>
+      <c r="N17" s="9">
+        <v>4</v>
+      </c>
+      <c r="O17" s="9">
+        <v>3</v>
+      </c>
+      <c r="P17" s="9">
+        <v>4</v>
+      </c>
+      <c r="Q17" s="9">
+        <v>2</v>
+      </c>
+      <c r="R17" s="9">
+        <v>4</v>
+      </c>
+      <c r="S17">
         <f t="shared" si="0"/>
-        <v/>
+        <v>3.5</v>
+      </c>
+      <c r="T17" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="18" spans="1:20" x14ac:dyDescent="0.3">
@@ -4125,17 +4197,33 @@
       <c r="J18" s="10" t="s">
         <v>131</v>
       </c>
-      <c r="K18" s="9"/>
-      <c r="L18" s="9"/>
-      <c r="M18" s="9"/>
-      <c r="N18" s="9"/>
-      <c r="O18" s="9"/>
-      <c r="P18" s="9"/>
-      <c r="Q18" s="9"/>
-      <c r="R18" s="9"/>
-      <c r="S18" t="str">
+      <c r="K18" s="9">
+        <v>5</v>
+      </c>
+      <c r="L18" s="9">
+        <v>4</v>
+      </c>
+      <c r="M18" s="9">
+        <v>4</v>
+      </c>
+      <c r="N18" s="9">
+        <v>5</v>
+      </c>
+      <c r="O18" s="9">
+        <v>4</v>
+      </c>
+      <c r="P18" s="9">
+        <v>5</v>
+      </c>
+      <c r="Q18" s="9">
+        <v>4</v>
+      </c>
+      <c r="R18" s="9">
+        <v>4</v>
+      </c>
+      <c r="S18">
         <f t="shared" si="0"/>
-        <v/>
+        <v>4.375</v>
       </c>
     </row>
     <row r="20" spans="1:20" x14ac:dyDescent="0.3">
@@ -4285,17 +4373,36 @@
       <c r="J22" s="10" t="s">
         <v>131</v>
       </c>
-      <c r="K22" s="9"/>
-      <c r="L22" s="9"/>
-      <c r="M22" s="9"/>
-      <c r="N22" s="9"/>
-      <c r="O22" s="9"/>
-      <c r="P22" s="9"/>
-      <c r="Q22" s="9"/>
-      <c r="R22" s="9"/>
-      <c r="S22" t="str">
+      <c r="K22" s="9">
+        <v>2</v>
+      </c>
+      <c r="L22" s="9">
+        <v>4</v>
+      </c>
+      <c r="M22" s="9">
+        <v>4</v>
+      </c>
+      <c r="N22" s="9">
+        <v>4</v>
+      </c>
+      <c r="O22" s="9">
+        <v>5</v>
+      </c>
+      <c r="P22" s="9">
+        <v>2</v>
+      </c>
+      <c r="Q22" s="9">
+        <v>2</v>
+      </c>
+      <c r="R22" s="9">
+        <v>4</v>
+      </c>
+      <c r="S22">
         <f t="shared" si="1"/>
-        <v/>
+        <v>3.375</v>
+      </c>
+      <c r="T22" t="s">
+        <v>162</v>
       </c>
     </row>
     <row r="23" spans="1:20" x14ac:dyDescent="0.3">
@@ -4326,17 +4433,36 @@
       <c r="J23" t="s">
         <v>131</v>
       </c>
-      <c r="K23" s="9"/>
-      <c r="L23" s="9"/>
-      <c r="M23" s="9"/>
-      <c r="N23" s="9"/>
-      <c r="O23" s="9"/>
-      <c r="P23" s="9"/>
-      <c r="Q23" s="9"/>
-      <c r="R23" s="9"/>
-      <c r="S23" t="str">
+      <c r="K23" s="9">
+        <v>4</v>
+      </c>
+      <c r="L23" s="9">
+        <v>3</v>
+      </c>
+      <c r="M23" s="9">
+        <v>4</v>
+      </c>
+      <c r="N23" s="9">
+        <v>4</v>
+      </c>
+      <c r="O23" s="9">
+        <v>3</v>
+      </c>
+      <c r="P23" s="9">
+        <v>2</v>
+      </c>
+      <c r="Q23" s="9">
+        <v>2</v>
+      </c>
+      <c r="R23" s="9">
+        <v>4</v>
+      </c>
+      <c r="S23">
         <f t="shared" si="1"/>
-        <v/>
+        <v>3.25</v>
+      </c>
+      <c r="T23" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="24" spans="1:20" x14ac:dyDescent="0.3">
@@ -4368,17 +4494,33 @@
       <c r="J24" s="10" t="s">
         <v>131</v>
       </c>
-      <c r="K24" s="9"/>
-      <c r="L24" s="9"/>
-      <c r="M24" s="9"/>
-      <c r="N24" s="9"/>
-      <c r="O24" s="9"/>
-      <c r="P24" s="9"/>
-      <c r="Q24" s="9"/>
-      <c r="R24" s="9"/>
-      <c r="S24" t="str">
+      <c r="K24" s="9">
+        <v>4</v>
+      </c>
+      <c r="L24" s="9">
+        <v>3</v>
+      </c>
+      <c r="M24" s="9">
+        <v>4</v>
+      </c>
+      <c r="N24" s="9">
+        <v>4</v>
+      </c>
+      <c r="O24" s="9">
+        <v>3</v>
+      </c>
+      <c r="P24" s="9">
+        <v>3</v>
+      </c>
+      <c r="Q24" s="9">
+        <v>4</v>
+      </c>
+      <c r="R24" s="9">
+        <v>3</v>
+      </c>
+      <c r="S24">
         <f t="shared" si="1"/>
-        <v/>
+        <v>3.5</v>
       </c>
     </row>
     <row r="25" spans="1:20" x14ac:dyDescent="0.3">
@@ -4451,17 +4593,33 @@
       <c r="J26" s="10" t="s">
         <v>131</v>
       </c>
-      <c r="K26" s="9"/>
-      <c r="L26" s="9"/>
-      <c r="M26" s="9"/>
-      <c r="N26" s="9"/>
-      <c r="O26" s="9"/>
-      <c r="P26" s="9"/>
-      <c r="Q26" s="9"/>
-      <c r="R26" s="9"/>
-      <c r="S26" t="str">
+      <c r="K26" s="9">
+        <v>3</v>
+      </c>
+      <c r="L26" s="9">
+        <v>5</v>
+      </c>
+      <c r="M26" s="9">
+        <v>4</v>
+      </c>
+      <c r="N26" s="9">
+        <v>4</v>
+      </c>
+      <c r="O26" s="9">
+        <v>5</v>
+      </c>
+      <c r="P26" s="9">
+        <v>3</v>
+      </c>
+      <c r="Q26" s="9">
+        <v>4</v>
+      </c>
+      <c r="R26" s="9">
+        <v>4</v>
+      </c>
+      <c r="S26">
         <f t="shared" si="1"/>
-        <v/>
+        <v>4</v>
       </c>
     </row>
     <row r="27" spans="1:20" x14ac:dyDescent="0.3">
@@ -4492,17 +4650,36 @@
       <c r="J27" t="s">
         <v>131</v>
       </c>
-      <c r="K27" s="9"/>
-      <c r="L27" s="9"/>
-      <c r="M27" s="9"/>
-      <c r="N27" s="9"/>
-      <c r="O27" s="9"/>
-      <c r="P27" s="9"/>
-      <c r="Q27" s="9"/>
-      <c r="R27" s="9"/>
-      <c r="S27" t="str">
+      <c r="K27" s="9">
+        <v>3</v>
+      </c>
+      <c r="L27" s="9">
+        <v>4</v>
+      </c>
+      <c r="M27" s="9">
+        <v>4</v>
+      </c>
+      <c r="N27" s="9">
+        <v>4</v>
+      </c>
+      <c r="O27" s="9">
+        <v>3</v>
+      </c>
+      <c r="P27" s="9">
+        <v>3</v>
+      </c>
+      <c r="Q27" s="9">
+        <v>2</v>
+      </c>
+      <c r="R27" s="9">
+        <v>4</v>
+      </c>
+      <c r="S27">
         <f t="shared" si="1"/>
-        <v/>
+        <v>3.375</v>
+      </c>
+      <c r="T27" t="s">
+        <v>159</v>
       </c>
     </row>
     <row r="28" spans="1:20" x14ac:dyDescent="0.3">
@@ -4534,17 +4711,36 @@
       <c r="J28" s="10" t="s">
         <v>131</v>
       </c>
-      <c r="K28" s="9"/>
-      <c r="L28" s="9"/>
-      <c r="M28" s="9"/>
-      <c r="N28" s="9"/>
-      <c r="O28" s="9"/>
-      <c r="P28" s="9"/>
-      <c r="Q28" s="9"/>
-      <c r="R28" s="9"/>
-      <c r="S28" t="str">
+      <c r="K28" s="9">
+        <v>4</v>
+      </c>
+      <c r="L28" s="9">
+        <v>4</v>
+      </c>
+      <c r="M28" s="9">
+        <v>4</v>
+      </c>
+      <c r="N28" s="9">
+        <v>4</v>
+      </c>
+      <c r="O28" s="9">
+        <v>3</v>
+      </c>
+      <c r="P28" s="9">
+        <v>3</v>
+      </c>
+      <c r="Q28" s="9">
+        <v>2</v>
+      </c>
+      <c r="R28" s="9">
+        <v>3</v>
+      </c>
+      <c r="S28">
         <f t="shared" si="1"/>
-        <v/>
+        <v>3.375</v>
+      </c>
+      <c r="T28" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="29" spans="1:20" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Task 2: replace FAILED TN Custom Media with TN settings and troubleshooting (22 chunks)
</commit_message>
<xml_diff>
--- a/doc_readiness_checklist.xlsx
+++ b/doc_readiness_checklist.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\AQCWT\OpenCode_Doc\APAI_Chat\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CF5B6D5-D258-4560-9532-A0D71112C962}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B7392B2-A088-4AD4-82C0-CD64E198642C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{BE8B64C7-7DD3-42E9-8432-DA4C4DC91B80}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{BE8B64C7-7DD3-42E9-8432-DA4C4DC91B80}"/>
   </bookViews>
   <sheets>
     <sheet name="All Documents – Status" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="498" uniqueCount="164">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="497" uniqueCount="164">
   <si>
     <t>ID</t>
   </si>
@@ -456,9 +456,6 @@
     <t>Tutorial – Impose v14: Lesson 26 - Number-Up Cut and Assemble</t>
   </si>
   <si>
-    <t>Technical Note – Proofing: TN Apogee Prepress 14 - Custom Media advanced mode</t>
-  </si>
-  <si>
     <t>Tutorial – QMS: QMS-Check-and-Double-Check</t>
   </si>
   <si>
@@ -532,6 +529,9 @@
   </si>
   <si>
     <t>C7=2: No troubleshooting scenarios for passkey failures or browser compatibility issues.</t>
+  </si>
+  <si>
+    <t>Technical Note - Proofing: TN Apogee Prepress 14 - settings and troubleshooting</t>
   </si>
 </sst>
 </file>
@@ -3612,7 +3612,7 @@
         <v>3.5</v>
       </c>
       <c r="T5" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="6" spans="1:20" x14ac:dyDescent="0.3">
@@ -3841,7 +3841,7 @@
     </row>
     <row r="11" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>138</v>
+        <v>163</v>
       </c>
       <c r="B11" t="s">
         <v>21</v>
@@ -3852,18 +3852,19 @@
       <c r="D11">
         <v>14</v>
       </c>
+      <c r="E11" s="2">
+        <v>46150.365972222222</v>
+      </c>
       <c r="F11" s="5" t="s">
-        <v>71</v>
+        <v>13</v>
       </c>
       <c r="G11">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="H11">
         <v>0</v>
       </c>
-      <c r="I11" s="6" t="s">
-        <v>71</v>
-      </c>
+      <c r="I11" s="6"/>
       <c r="J11" t="s">
         <v>131</v>
       </c>
@@ -3875,14 +3876,10 @@
       <c r="P11" s="9"/>
       <c r="Q11" s="9"/>
       <c r="R11" s="9"/>
-      <c r="S11" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
     </row>
     <row r="12" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A12" s="10" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B12" s="10" t="s">
         <v>21</v>
@@ -3924,7 +3921,7 @@
     </row>
     <row r="13" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B13" t="s">
         <v>21</v>
@@ -3965,7 +3962,7 @@
     </row>
     <row r="14" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A14" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B14" s="10" t="s">
         <v>21</v>
@@ -4007,7 +4004,7 @@
     </row>
     <row r="15" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B15" t="s">
         <v>21</v>
@@ -4048,7 +4045,7 @@
     </row>
     <row r="16" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A16" s="10" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B16" s="10" t="s">
         <v>101</v>
@@ -4072,7 +4069,7 @@
         <v>0</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="J16" s="10" t="s">
         <v>131</v>
@@ -4108,7 +4105,7 @@
     </row>
     <row r="17" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B17" t="s">
         <v>101</v>
@@ -4163,12 +4160,12 @@
         <v>3.5</v>
       </c>
       <c r="T17" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="18" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A18" s="10" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B18" s="10" t="s">
         <v>101</v>
@@ -4192,7 +4189,7 @@
         <v>0</v>
       </c>
       <c r="I18" s="10" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="J18" s="10" t="s">
         <v>131</v>
@@ -4228,7 +4225,7 @@
     </row>
     <row r="20" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A20" s="10" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B20" s="10" t="s">
         <v>11</v>
@@ -4284,12 +4281,12 @@
         <v>3.375</v>
       </c>
       <c r="T20" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="21" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B21" t="s">
         <v>11</v>
@@ -4346,7 +4343,7 @@
     </row>
     <row r="22" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A22" s="10" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B22" s="10" t="s">
         <v>21</v>
@@ -4402,12 +4399,12 @@
         <v>3.375</v>
       </c>
       <c r="T22" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="23" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B23" t="s">
         <v>21</v>
@@ -4462,12 +4459,12 @@
         <v>3.25</v>
       </c>
       <c r="T23" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="24" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A24" s="10" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B24" s="10" t="s">
         <v>21</v>
@@ -4525,7 +4522,7 @@
     </row>
     <row r="25" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B25" t="s">
         <v>21</v>
@@ -4566,7 +4563,7 @@
     </row>
     <row r="26" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A26" s="10" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B26" s="10" t="s">
         <v>21</v>
@@ -4624,7 +4621,7 @@
     </row>
     <row r="27" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B27" t="s">
         <v>101</v>
@@ -4679,12 +4676,12 @@
         <v>3.375</v>
       </c>
       <c r="T27" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="28" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A28" s="10" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B28" s="10" t="s">
         <v>101</v>
@@ -4740,12 +4737,12 @@
         <v>3.375</v>
       </c>
       <c r="T28" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="29" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A29" s="14" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B29" s="14"/>
       <c r="C29" s="14"/>

</xml_diff>

<commit_message>
Checklist: replace ? markers with star for all 24 sampled docs, clear TN Custom Media
</commit_message>
<xml_diff>
--- a/doc_readiness_checklist.xlsx
+++ b/doc_readiness_checklist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\AQCWT\OpenCode_Doc\APAI_Chat\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B7392B2-A088-4AD4-82C0-CD64E198642C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF931B3E-1FA1-4C33-8D21-500D2F26ED9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{BE8B64C7-7DD3-42E9-8432-DA4C4DC91B80}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="497" uniqueCount="164">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="506" uniqueCount="173">
   <si>
     <t>ID</t>
   </si>
@@ -84,454 +84,481 @@
     <t>COMPLETED</t>
   </si>
   <si>
+    <t>Apogee-Impose-Trick_Changing-the-Apogee-Impose-View</t>
+  </si>
+  <si>
+    <t>Apogee-Impose-Trick_Folding-Direction-Arrow</t>
+  </si>
+  <si>
+    <t>Apogee-InkDrive-Trick_Accurate-CIP3-Presets</t>
+  </si>
+  <si>
+    <t>testfile</t>
+  </si>
+  <si>
+    <t>OTHER</t>
+  </si>
+  <si>
+    <t>Apogee_Prepress_OLH_14.0.2_en-US</t>
+  </si>
+  <si>
+    <t>PREPRESS</t>
+  </si>
+  <si>
+    <t>Apogee-Proofing-Trick_Customized-White-Point-with-Absolute-Colorimetric-Proofing</t>
+  </si>
+  <si>
+    <t>Apogee-Proofing-Trick_GDIProofer-and-Split4ProofApogee</t>
+  </si>
+  <si>
+    <t>Apogee-Tips_Apogee-Prepress-with-Packaging-Pack</t>
+  </si>
+  <si>
+    <t>Apogee-Tips_JDF-Integration-Explained-in-a-Nutshell</t>
+  </si>
+  <si>
+    <t>Apogee-Tips_Packaging-Arbitrary-Rotation</t>
+  </si>
+  <si>
+    <t>Apogee-Tips_QuickProof-from-the-Raster-Preview</t>
+  </si>
+  <si>
+    <t>Apogee-Tips_Saving-Money-with-SolidTune</t>
+  </si>
+  <si>
+    <t>Apogee-Tips_Versioning</t>
+  </si>
+  <si>
+    <t>Apogee-Tips_WebApproval-A-Fully-Integrated-Softproof-Solution</t>
+  </si>
+  <si>
+    <t>Apogee-Trick_Apogee-DQS</t>
+  </si>
+  <si>
+    <t>Apogee-Trick_Automate-Job-Creation-with-ApoXML</t>
+  </si>
+  <si>
+    <t>Apogee-Trick_Auto-Route-PDF-Files-with-Automate-TP</t>
+  </si>
+  <si>
+    <t>Apogee-Trick_Client-Customization</t>
+  </si>
+  <si>
+    <t>Apogee-Trick_Customized-White-Point-with-Absolute-Colorimetric-Proofing</t>
+  </si>
+  <si>
+    <t>Apogee-Trick_Exporting-of-PDFs</t>
+  </si>
+  <si>
+    <t>Apogee-Trick_Offline-Jobs</t>
+  </si>
+  <si>
+    <t>Apogee-Trick_Packaging-and-Automation</t>
+  </si>
+  <si>
+    <t>The Essential Role of Virus Scanning and Tuning</t>
+  </si>
+  <si>
+    <t>APAI Chat - About This Assistant</t>
+  </si>
+  <si>
+    <t>REFERENCE_GUIDE</t>
+  </si>
+  <si>
+    <t>Apogee Prepress_QMS_OLH</t>
+  </si>
+  <si>
+    <t>Apogee_Impose_RG_14.0.1_en-US</t>
+  </si>
+  <si>
+    <t>ApogeeColor InkLimitation target</t>
+  </si>
+  <si>
+    <t>TUTORIAL</t>
+  </si>
+  <si>
+    <t>Basic Administrative Tasks</t>
+  </si>
+  <si>
+    <t>Creating and Editing Job Tickets</t>
+  </si>
+  <si>
+    <t>Creating and Managing Device Borders</t>
+  </si>
+  <si>
+    <t>Creating and Managing Linearization, Calibration and Simulation Curves</t>
+  </si>
+  <si>
+    <t>Creating and managing Web Growth Profiles</t>
+  </si>
+  <si>
+    <t>Creating Hot Tickets</t>
+  </si>
+  <si>
+    <t>Editing Hot Tickets</t>
+  </si>
+  <si>
+    <t>Ink Limit target</t>
+  </si>
+  <si>
+    <t>Job Housekeeping</t>
+  </si>
+  <si>
+    <t>Lesson 26 - Number-Up Cut and Assemble</t>
+  </si>
+  <si>
+    <t>Lesson 27 - Mixed Assemblies with Auto Impose</t>
+  </si>
+  <si>
+    <t>Proofing-Contract-Proofing</t>
+  </si>
+  <si>
+    <t>QMS-Check-and-Double-Check</t>
+  </si>
+  <si>
+    <t>QMS-History-Tracking</t>
+  </si>
+  <si>
+    <t>QMS-Improve-Quality</t>
+  </si>
+  <si>
+    <t>Quick Tour</t>
+  </si>
+  <si>
+    <t>TN Apogee Prepress 14 - Custom Media advanced mode</t>
+  </si>
+  <si>
+    <t>FAILED</t>
+  </si>
+  <si>
+    <t>FAILED – re-upload needed</t>
+  </si>
+  <si>
+    <t>TN Apogee Prepress 14 - Custom Media Simple mode</t>
+  </si>
+  <si>
+    <t>TN Apogee Prepress 14 - Measurement devices</t>
+  </si>
+  <si>
+    <t>TN Apogee Prepress 14 - Profiling for Proofers</t>
+  </si>
+  <si>
+    <t>TN Apogee Prepress 14 - Proof validation and certification</t>
+  </si>
+  <si>
+    <t>TN Apogee Prepress 14 - settings and troubleshooting</t>
+  </si>
+  <si>
+    <t>TN Apogee Prepress v14 - Calibration follow up</t>
+  </si>
+  <si>
+    <t>TN Apogee Prepress v14 - Hardcopy Proofing Toolkit</t>
+  </si>
+  <si>
+    <t>TN Apogee Prepress v14 - Standardization to ISO</t>
+  </si>
+  <si>
+    <t>Working with Filters</t>
+  </si>
+  <si>
+    <t>Working with Hot Tickets</t>
+  </si>
+  <si>
+    <t>Working with Job Tickets</t>
+  </si>
+  <si>
+    <t>Working with Messages</t>
+  </si>
+  <si>
+    <t>Working with Split for Proof</t>
+  </si>
+  <si>
+    <t>ApogeePrepress_ImpTut_14.0_en-US</t>
+  </si>
+  <si>
+    <t>Advanced Job Management</t>
+  </si>
+  <si>
+    <t>Apogee Preflight</t>
+  </si>
+  <si>
+    <t>Exporting Documents</t>
+  </si>
+  <si>
+    <t>Interactive Editing</t>
+  </si>
+  <si>
+    <t>Separation Handling</t>
+  </si>
+  <si>
+    <t>Trapping</t>
+  </si>
+  <si>
+    <t>PARTIALLY_COMPLETED</t>
+  </si>
+  <si>
+    <t>Partial – check failed images</t>
+  </si>
+  <si>
+    <t>Versioning - Basic</t>
+  </si>
+  <si>
+    <t>PrintSphere_OLH_en-US_draft01</t>
+  </si>
+  <si>
+    <t>ProductionCenter_UG_14.0_en-US</t>
+  </si>
+  <si>
+    <t>PRODUCTION_CENTER</t>
+  </si>
+  <si>
+    <t>ProductionCenter-Tips_Displaying-MISID-in-WebApproval</t>
+  </si>
+  <si>
+    <t>ProductionCenter-Tips_ECO3-Production-Dashboard</t>
+  </si>
+  <si>
+    <t>ProductionCenter-Tips_Enhanced-Collaboration</t>
+  </si>
+  <si>
+    <t>ProductionCenter-Tips_Message-Configuration</t>
+  </si>
+  <si>
+    <t>ProductionCenter-Tips_Passkeys</t>
+  </si>
+  <si>
+    <t>ProductionCenter-Tips_Supplementary-Files</t>
+  </si>
+  <si>
+    <t>Approve and reject pages</t>
+  </si>
+  <si>
+    <t>Print-Buyer Company - Managing Company &amp; Users</t>
+  </si>
+  <si>
+    <t>Printer Company - Managing Companies &amp; Users</t>
+  </si>
+  <si>
+    <t>Upload and assign files</t>
+  </si>
+  <si>
+    <t>Working with WebFlow</t>
+  </si>
+  <si>
+    <t>APAI Chat – Phase 1: Documentation Readiness Checklist (Section 5)</t>
+  </si>
+  <si>
+    <t>Scoring: 1=Unusable  2=Major rework  3=Usable with gaps  4=Good  5=Excellent (RAG-ready)     |    AUTO = populated from API     |    ★ = selected sample</t>
+  </si>
+  <si>
+    <t>Ingestion Flag</t>
+  </si>
+  <si>
+    <t>Sample?</t>
+  </si>
+  <si>
+    <t>1. Structural Clarity</t>
+  </si>
+  <si>
+    <t>2. Self-Containment</t>
+  </si>
+  <si>
+    <t>3. Explicit Context</t>
+  </si>
+  <si>
+    <t>4. Term Consistency</t>
+  </si>
+  <si>
+    <t>5. Text/Image Ratio</t>
+  </si>
+  <si>
+    <t>6. Procedure Clarity</t>
+  </si>
+  <si>
+    <t>7. Error Proximity</t>
+  </si>
+  <si>
+    <t>8. Chunk-Friendliness</t>
+  </si>
+  <si>
+    <t>Avg Score</t>
+  </si>
+  <si>
+    <t>Priority Action</t>
+  </si>
+  <si>
+    <t>Tips &amp; Tricks – Impose: Apogee-Impose-Trick_Automatic-Page-Numbering</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>Tips &amp; Tricks – Prepress: Apogee-Trick_Apogee-DQS</t>
+  </si>
+  <si>
+    <t>Online Help – Prepress: Apogee_Prepress_OLH_14.0.2_en-US</t>
+  </si>
+  <si>
+    <t>Reference Guide – Impose: Apogee_Impose_RG_14.0.1_en-US</t>
+  </si>
+  <si>
+    <t>Reference Guide – QMS: Apogee Prepress_QMS_OLH</t>
+  </si>
+  <si>
+    <t>Tutorial – Prepress v14: Basic Administrative Tasks</t>
+  </si>
+  <si>
+    <t>Tutorial – Impose v14: Lesson 26 - Number-Up Cut and Assemble</t>
+  </si>
+  <si>
+    <t>Tutorial – QMS: QMS-Check-and-Double-Check</t>
+  </si>
+  <si>
+    <t>Tutorial – Proofing: Proofing-Contract-Proofing</t>
+  </si>
+  <si>
+    <t>Tutorial – Prepress v15: Advanced Job Management</t>
+  </si>
+  <si>
+    <t>Online Help – PrintSphere: PrintSphere_OLH_en-US_draft01</t>
+  </si>
+  <si>
+    <t>User Guide – ProductionCenter: ProductionCenter_UG_14.0_en-US</t>
+  </si>
+  <si>
+    <t>Partial – check images</t>
+  </si>
+  <si>
+    <t>Tips &amp; Tricks – ProductionCenter: ProductionCenter-Tips_Passkeys</t>
+  </si>
+  <si>
+    <t>Tutorial – ProductionCenter: Approve and reject pages</t>
+  </si>
+  <si>
+    <t>⚠ Documents scoring ≤2 on any criterion need remediation before launch (per Section 5 of AI Testing &amp; Evaluation Plan v1.4)</t>
+  </si>
+  <si>
+    <t>Tips &amp; Tricks – Impose (Folding): Apogee-Impose-Trick_Folding-Direction-Arrow</t>
+  </si>
+  <si>
+    <t>Tips &amp; Tricks – InkDrive: Apogee-InkDrive-Trick_Accurate-CIP3-Presets</t>
+  </si>
+  <si>
+    <t>Tips &amp; Tricks – Proofing: Apogee-Proofing-Trick_GDIProofer-and-Split4ProofApogee</t>
+  </si>
+  <si>
+    <t>Tips &amp; Tricks – Packaging: Apogee-Tips_Apogee-Prepress-with-Packaging-Pack</t>
+  </si>
+  <si>
+    <t>Tips &amp; Tricks – WebApproval: Apogee-Tips_WebApproval-A-Fully-Integrated-Softproof-Solution</t>
+  </si>
+  <si>
+    <t>Tips &amp; Tricks – Automation: Apogee-Trick_Auto-Route-PDF-Files-with-Automate-TP</t>
+  </si>
+  <si>
+    <t>Tips &amp; Tricks – General: The Essential Role of Virus Scanning and Tuning</t>
+  </si>
+  <si>
+    <t>Tips &amp; Tricks – ProductionCenter Dashboard: ProductionCenter-Tips_ECO3-Production-Dashboard</t>
+  </si>
+  <si>
+    <t>Tips &amp; Tricks – ProductionCenter Collaboration: ProductionCenter-Tips_Enhanced-Collaboration</t>
+  </si>
+  <si>
+    <t>Criterion 5 (Text/Image Ratio=2): Key fold direction information relies heavily on images; add text description of arrow direction.</t>
+  </si>
+  <si>
+    <t>C7=2: No troubleshooting content for annotation or notification failures.</t>
+  </si>
+  <si>
+    <t>C7=2: No troubleshooting content for data access or dashboard issues.</t>
+  </si>
+  <si>
+    <t>C6=2: Overview only; links to external tutorials but no procedural steps in document. C7=2: No troubleshooting content.</t>
+  </si>
+  <si>
+    <t>C6=2: No procedure steps for DQS activation or configuration. C7=2: No troubleshooting content.</t>
+  </si>
+  <si>
+    <t>C1=2: No internal section headings within body text. C6=2: Feature description only - no setup or usage steps included. C7=2: No error or troubleshooting content.</t>
+  </si>
+  <si>
+    <t>C7=2: No troubleshooting scenarios for passkey failures or browser compatibility issues.</t>
+  </si>
+  <si>
+    <t>Technical Note - Proofing: TN Apogee Prepress 14 - settings and troubleshooting</t>
+  </si>
+  <si>
     <t>★ 124</t>
   </si>
   <si>
-    <t>Apogee-Impose-Trick_Changing-the-Apogee-Impose-View</t>
-  </si>
-  <si>
-    <t>Apogee-Impose-Trick_Folding-Direction-Arrow</t>
-  </si>
-  <si>
-    <t>Apogee-InkDrive-Trick_Accurate-CIP3-Presets</t>
-  </si>
-  <si>
-    <t>testfile</t>
-  </si>
-  <si>
-    <t>OTHER</t>
-  </si>
-  <si>
-    <t>Apogee_Prepress_OLH_14.0.2_en-US</t>
-  </si>
-  <si>
-    <t>PREPRESS</t>
+    <t>★ 126</t>
+  </si>
+  <si>
+    <t>★ 127</t>
   </si>
   <si>
     <t>★ 39</t>
   </si>
   <si>
-    <t>Apogee-Proofing-Trick_Customized-White-Point-with-Absolute-Colorimetric-Proofing</t>
-  </si>
-  <si>
-    <t>Apogee-Proofing-Trick_GDIProofer-and-Split4ProofApogee</t>
-  </si>
-  <si>
-    <t>Apogee-Tips_Apogee-Prepress-with-Packaging-Pack</t>
-  </si>
-  <si>
-    <t>Apogee-Tips_JDF-Integration-Explained-in-a-Nutshell</t>
-  </si>
-  <si>
-    <t>Apogee-Tips_Packaging-Arbitrary-Rotation</t>
-  </si>
-  <si>
-    <t>Apogee-Tips_QuickProof-from-the-Raster-Preview</t>
-  </si>
-  <si>
-    <t>Apogee-Tips_Saving-Money-with-SolidTune</t>
-  </si>
-  <si>
-    <t>Apogee-Tips_Versioning</t>
-  </si>
-  <si>
-    <t>Apogee-Tips_WebApproval-A-Fully-Integrated-Softproof-Solution</t>
-  </si>
-  <si>
-    <t>Apogee-Trick_Apogee-DQS</t>
+    <t>★ 86</t>
+  </si>
+  <si>
+    <t>★ 87</t>
+  </si>
+  <si>
+    <t>★ 75</t>
   </si>
   <si>
     <t>★ 76</t>
   </si>
   <si>
-    <t>Apogee-Trick_Automate-Job-Creation-with-ApoXML</t>
-  </si>
-  <si>
-    <t>Apogee-Trick_Auto-Route-PDF-Files-with-Automate-TP</t>
-  </si>
-  <si>
-    <t>Apogee-Trick_Client-Customization</t>
-  </si>
-  <si>
-    <t>Apogee-Trick_Customized-White-Point-with-Absolute-Colorimetric-Proofing</t>
-  </si>
-  <si>
-    <t>Apogee-Trick_Exporting-of-PDFs</t>
-  </si>
-  <si>
-    <t>Apogee-Trick_Offline-Jobs</t>
-  </si>
-  <si>
-    <t>Apogee-Trick_Packaging-and-Automation</t>
-  </si>
-  <si>
-    <t>The Essential Role of Virus Scanning and Tuning</t>
-  </si>
-  <si>
-    <t>APAI Chat - About This Assistant</t>
-  </si>
-  <si>
-    <t>REFERENCE_GUIDE</t>
-  </si>
-  <si>
-    <t>Apogee Prepress_QMS_OLH</t>
+    <t>★ 78</t>
+  </si>
+  <si>
+    <t>★ 84</t>
   </si>
   <si>
     <t>★ 43</t>
   </si>
   <si>
-    <t>Apogee_Impose_RG_14.0.1_en-US</t>
-  </si>
-  <si>
     <t>★ 62</t>
   </si>
   <si>
-    <t>ApogeeColor InkLimitation target</t>
-  </si>
-  <si>
-    <t>TUTORIAL</t>
-  </si>
-  <si>
-    <t>Basic Administrative Tasks</t>
-  </si>
-  <si>
     <t>★ 98</t>
   </si>
   <si>
-    <t>Creating and Editing Job Tickets</t>
-  </si>
-  <si>
-    <t>Creating and Managing Device Borders</t>
-  </si>
-  <si>
-    <t>Creating and Managing Linearization, Calibration and Simulation Curves</t>
-  </si>
-  <si>
-    <t>Creating and managing Web Growth Profiles</t>
-  </si>
-  <si>
-    <t>Creating Hot Tickets</t>
-  </si>
-  <si>
-    <t>Editing Hot Tickets</t>
-  </si>
-  <si>
-    <t>Ink Limit target</t>
-  </si>
-  <si>
-    <t>Job Housekeeping</t>
-  </si>
-  <si>
-    <t>Lesson 26 - Number-Up Cut and Assemble</t>
-  </si>
-  <si>
     <t>★ 95</t>
   </si>
   <si>
-    <t>Lesson 27 - Mixed Assemblies with Auto Impose</t>
-  </si>
-  <si>
-    <t>Proofing-Contract-Proofing</t>
-  </si>
-  <si>
     <t>★ 44</t>
   </si>
   <si>
-    <t>QMS-Check-and-Double-Check</t>
-  </si>
-  <si>
     <t>★ 45</t>
   </si>
   <si>
-    <t>QMS-History-Tracking</t>
-  </si>
-  <si>
-    <t>QMS-Improve-Quality</t>
-  </si>
-  <si>
-    <t>Quick Tour</t>
-  </si>
-  <si>
-    <t>TN Apogee Prepress 14 - Custom Media advanced mode</t>
-  </si>
-  <si>
-    <t>FAILED</t>
-  </si>
-  <si>
-    <t>FAILED – re-upload needed</t>
-  </si>
-  <si>
-    <t>★ 53</t>
-  </si>
-  <si>
-    <t>TN Apogee Prepress 14 - Custom Media Simple mode</t>
-  </si>
-  <si>
-    <t>TN Apogee Prepress 14 - Measurement devices</t>
-  </si>
-  <si>
-    <t>TN Apogee Prepress 14 - Profiling for Proofers</t>
-  </si>
-  <si>
-    <t>TN Apogee Prepress 14 - Proof validation and certification</t>
-  </si>
-  <si>
-    <t>TN Apogee Prepress 14 - settings and troubleshooting</t>
-  </si>
-  <si>
-    <t>TN Apogee Prepress v14 - Calibration follow up</t>
-  </si>
-  <si>
-    <t>TN Apogee Prepress v14 - Hardcopy Proofing Toolkit</t>
-  </si>
-  <si>
-    <t>TN Apogee Prepress v14 - Standardization to ISO</t>
-  </si>
-  <si>
-    <t>Working with Filters</t>
-  </si>
-  <si>
-    <t>Working with Hot Tickets</t>
-  </si>
-  <si>
-    <t>Working with Job Tickets</t>
-  </si>
-  <si>
-    <t>Working with Messages</t>
-  </si>
-  <si>
-    <t>Working with Split for Proof</t>
-  </si>
-  <si>
-    <t>ApogeePrepress_ImpTut_14.0_en-US</t>
-  </si>
-  <si>
-    <t>Advanced Job Management</t>
+    <t>★ 58</t>
   </si>
   <si>
     <t>★ 117</t>
   </si>
   <si>
-    <t>Apogee Preflight</t>
-  </si>
-  <si>
-    <t>Exporting Documents</t>
-  </si>
-  <si>
-    <t>Interactive Editing</t>
-  </si>
-  <si>
-    <t>Separation Handling</t>
-  </si>
-  <si>
-    <t>Trapping</t>
-  </si>
-  <si>
-    <t>PARTIALLY_COMPLETED</t>
-  </si>
-  <si>
-    <t>Partial – check failed images</t>
-  </si>
-  <si>
-    <t>Versioning - Basic</t>
-  </si>
-  <si>
-    <t>PrintSphere_OLH_en-US_draft01</t>
-  </si>
-  <si>
     <t>★ 48</t>
   </si>
   <si>
-    <t>ProductionCenter_UG_14.0_en-US</t>
-  </si>
-  <si>
-    <t>PRODUCTION_CENTER</t>
-  </si>
-  <si>
     <t>★ 38</t>
   </si>
   <si>
-    <t>ProductionCenter-Tips_Displaying-MISID-in-WebApproval</t>
-  </si>
-  <si>
-    <t>ProductionCenter-Tips_ECO3-Production-Dashboard</t>
-  </si>
-  <si>
-    <t>ProductionCenter-Tips_Enhanced-Collaboration</t>
-  </si>
-  <si>
-    <t>ProductionCenter-Tips_Message-Configuration</t>
-  </si>
-  <si>
-    <t>ProductionCenter-Tips_Passkeys</t>
+    <t>★ 64</t>
+  </si>
+  <si>
+    <t>★ 71</t>
   </si>
   <si>
     <t>★ 67</t>
   </si>
   <si>
-    <t>ProductionCenter-Tips_Supplementary-Files</t>
-  </si>
-  <si>
-    <t>Approve and reject pages</t>
-  </si>
-  <si>
     <t>★ 116</t>
-  </si>
-  <si>
-    <t>Print-Buyer Company - Managing Company &amp; Users</t>
-  </si>
-  <si>
-    <t>Printer Company - Managing Companies &amp; Users</t>
-  </si>
-  <si>
-    <t>Upload and assign files</t>
-  </si>
-  <si>
-    <t>Working with WebFlow</t>
-  </si>
-  <si>
-    <t>APAI Chat – Phase 1: Documentation Readiness Checklist (Section 5)</t>
-  </si>
-  <si>
-    <t>Scoring: 1=Unusable  2=Major rework  3=Usable with gaps  4=Good  5=Excellent (RAG-ready)     |    AUTO = populated from API     |    ★ = selected sample</t>
-  </si>
-  <si>
-    <t>Ingestion Flag</t>
-  </si>
-  <si>
-    <t>Sample?</t>
-  </si>
-  <si>
-    <t>1. Structural Clarity</t>
-  </si>
-  <si>
-    <t>2. Self-Containment</t>
-  </si>
-  <si>
-    <t>3. Explicit Context</t>
-  </si>
-  <si>
-    <t>4. Term Consistency</t>
-  </si>
-  <si>
-    <t>5. Text/Image Ratio</t>
-  </si>
-  <si>
-    <t>6. Procedure Clarity</t>
-  </si>
-  <si>
-    <t>7. Error Proximity</t>
-  </si>
-  <si>
-    <t>8. Chunk-Friendliness</t>
-  </si>
-  <si>
-    <t>Avg Score</t>
-  </si>
-  <si>
-    <t>Priority Action</t>
-  </si>
-  <si>
-    <t>Tips &amp; Tricks – Impose: Apogee-Impose-Trick_Automatic-Page-Numbering</t>
-  </si>
-  <si>
-    <t>Yes</t>
-  </si>
-  <si>
-    <t>Tips &amp; Tricks – Prepress: Apogee-Trick_Apogee-DQS</t>
-  </si>
-  <si>
-    <t>Online Help – Prepress: Apogee_Prepress_OLH_14.0.2_en-US</t>
-  </si>
-  <si>
-    <t>Reference Guide – Impose: Apogee_Impose_RG_14.0.1_en-US</t>
-  </si>
-  <si>
-    <t>Reference Guide – QMS: Apogee Prepress_QMS_OLH</t>
-  </si>
-  <si>
-    <t>Tutorial – Prepress v14: Basic Administrative Tasks</t>
-  </si>
-  <si>
-    <t>Tutorial – Impose v14: Lesson 26 - Number-Up Cut and Assemble</t>
-  </si>
-  <si>
-    <t>Tutorial – QMS: QMS-Check-and-Double-Check</t>
-  </si>
-  <si>
-    <t>Tutorial – Proofing: Proofing-Contract-Proofing</t>
-  </si>
-  <si>
-    <t>Tutorial – Prepress v15: Advanced Job Management</t>
-  </si>
-  <si>
-    <t>Online Help – PrintSphere: PrintSphere_OLH_en-US_draft01</t>
-  </si>
-  <si>
-    <t>User Guide – ProductionCenter: ProductionCenter_UG_14.0_en-US</t>
-  </si>
-  <si>
-    <t>Partial – check images</t>
-  </si>
-  <si>
-    <t>Tips &amp; Tricks – ProductionCenter: ProductionCenter-Tips_Passkeys</t>
-  </si>
-  <si>
-    <t>Tutorial – ProductionCenter: Approve and reject pages</t>
-  </si>
-  <si>
-    <t>⚠ Documents scoring ≤2 on any criterion need remediation before launch (per Section 5 of AI Testing &amp; Evaluation Plan v1.4)</t>
-  </si>
-  <si>
-    <t>Tips &amp; Tricks – Impose (Folding): Apogee-Impose-Trick_Folding-Direction-Arrow</t>
-  </si>
-  <si>
-    <t>Tips &amp; Tricks – InkDrive: Apogee-InkDrive-Trick_Accurate-CIP3-Presets</t>
-  </si>
-  <si>
-    <t>Tips &amp; Tricks – Proofing: Apogee-Proofing-Trick_GDIProofer-and-Split4ProofApogee</t>
-  </si>
-  <si>
-    <t>Tips &amp; Tricks – Packaging: Apogee-Tips_Apogee-Prepress-with-Packaging-Pack</t>
-  </si>
-  <si>
-    <t>Tips &amp; Tricks – WebApproval: Apogee-Tips_WebApproval-A-Fully-Integrated-Softproof-Solution</t>
-  </si>
-  <si>
-    <t>Tips &amp; Tricks – Automation: Apogee-Trick_Auto-Route-PDF-Files-with-Automate-TP</t>
-  </si>
-  <si>
-    <t>Tips &amp; Tricks – General: The Essential Role of Virus Scanning and Tuning</t>
-  </si>
-  <si>
-    <t>Tips &amp; Tricks – ProductionCenter Dashboard: ProductionCenter-Tips_ECO3-Production-Dashboard</t>
-  </si>
-  <si>
-    <t>Tips &amp; Tricks – ProductionCenter Collaboration: ProductionCenter-Tips_Enhanced-Collaboration</t>
-  </si>
-  <si>
-    <t>Criterion 5 (Text/Image Ratio=2): Key fold direction information relies heavily on images; add text description of arrow direction.</t>
-  </si>
-  <si>
-    <t>C7=2: No troubleshooting content for annotation or notification failures.</t>
-  </si>
-  <si>
-    <t>C7=2: No troubleshooting content for data access or dashboard issues.</t>
-  </si>
-  <si>
-    <t>C6=2: Overview only; links to external tutorials but no procedural steps in document. C7=2: No troubleshooting content.</t>
-  </si>
-  <si>
-    <t>C6=2: No procedure steps for DQS activation or configuration. C7=2: No troubleshooting content.</t>
-  </si>
-  <si>
-    <t>C1=2: No internal section headings within body text. C6=2: Feature description only - no setup or usage steps included. C7=2: No error or troubleshooting content.</t>
-  </si>
-  <si>
-    <t>C7=2: No troubleshooting scenarios for passkey failures or browser compatibility issues.</t>
-  </si>
-  <si>
-    <t>Technical Note - Proofing: TN Apogee Prepress 14 - settings and troubleshooting</t>
   </si>
 </sst>
 </file>
@@ -1060,7 +1087,7 @@
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>14</v>
+        <v>149</v>
       </c>
       <c r="B2" t="s">
         <v>10</v>
@@ -1092,7 +1119,7 @@
         <v>125</v>
       </c>
       <c r="B3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C3" t="s">
         <v>11</v>
@@ -1117,11 +1144,11 @@
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A4">
-        <v>126</v>
+      <c r="A4" t="s">
+        <v>150</v>
       </c>
       <c r="B4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C4" t="s">
         <v>11</v>
@@ -1146,11 +1173,11 @@
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A5">
-        <v>127</v>
+      <c r="A5" t="s">
+        <v>151</v>
       </c>
       <c r="B5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C5" t="s">
         <v>11</v>
@@ -1179,13 +1206,13 @@
         <v>36</v>
       </c>
       <c r="B6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" t="s">
         <v>18</v>
       </c>
-      <c r="C6" t="s">
-        <v>19</v>
-      </c>
       <c r="D6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E6">
         <v>0.1</v>
@@ -1205,16 +1232,16 @@
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
-        <v>22</v>
+        <v>152</v>
       </c>
       <c r="B7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C7" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D7" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E7">
         <v>14</v>
@@ -1237,13 +1264,13 @@
         <v>85</v>
       </c>
       <c r="B8" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D8" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E8">
         <v>14</v>
@@ -1262,17 +1289,17 @@
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A9">
-        <v>86</v>
+      <c r="A9" t="s">
+        <v>153</v>
       </c>
       <c r="B9" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C9" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D9" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E9">
         <v>14</v>
@@ -1291,17 +1318,17 @@
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A10">
-        <v>87</v>
+      <c r="A10" t="s">
+        <v>154</v>
       </c>
       <c r="B10" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D10" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E10">
         <v>14</v>
@@ -1324,13 +1351,13 @@
         <v>88</v>
       </c>
       <c r="B11" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C11" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E11">
         <v>14</v>
@@ -1353,13 +1380,13 @@
         <v>89</v>
       </c>
       <c r="B12" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D12" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E12">
         <v>14</v>
@@ -1382,13 +1409,13 @@
         <v>90</v>
       </c>
       <c r="B13" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C13" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D13" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E13">
         <v>14</v>
@@ -1411,13 +1438,13 @@
         <v>91</v>
       </c>
       <c r="B14" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C14" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D14" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E14">
         <v>14</v>
@@ -1440,13 +1467,13 @@
         <v>92</v>
       </c>
       <c r="B15" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C15" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D15" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E15">
         <v>14</v>
@@ -1465,17 +1492,17 @@
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16">
-        <v>75</v>
+      <c r="A16" t="s">
+        <v>155</v>
       </c>
       <c r="B16" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C16" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D16" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E16">
         <v>14</v>
@@ -1495,16 +1522,16 @@
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
-        <v>33</v>
+        <v>156</v>
       </c>
       <c r="B17" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C17" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D17" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E17">
         <v>14</v>
@@ -1527,13 +1554,13 @@
         <v>77</v>
       </c>
       <c r="B18" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C18" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D18" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E18">
         <v>14</v>
@@ -1552,17 +1579,17 @@
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A19">
-        <v>78</v>
+      <c r="A19" t="s">
+        <v>157</v>
       </c>
       <c r="B19" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="C19" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D19" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E19">
         <v>14</v>
@@ -1585,13 +1612,13 @@
         <v>79</v>
       </c>
       <c r="B20" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C20" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D20" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E20">
         <v>14</v>
@@ -1614,13 +1641,13 @@
         <v>80</v>
       </c>
       <c r="B21" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="C21" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D21" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E21">
         <v>14</v>
@@ -1643,13 +1670,13 @@
         <v>81</v>
       </c>
       <c r="B22" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="C22" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D22" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E22">
         <v>14</v>
@@ -1672,13 +1699,13 @@
         <v>82</v>
       </c>
       <c r="B23" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C23" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D23" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E23">
         <v>14</v>
@@ -1701,13 +1728,13 @@
         <v>83</v>
       </c>
       <c r="B24" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C24" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D24" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E24">
         <v>14</v>
@@ -1726,17 +1753,17 @@
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A25">
-        <v>84</v>
+      <c r="A25" t="s">
+        <v>158</v>
       </c>
       <c r="B25" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C25" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D25" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E25">
         <v>14</v>
@@ -1759,13 +1786,13 @@
         <v>27</v>
       </c>
       <c r="B26" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="C26" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D26" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="F26" s="2">
         <v>46141.494444444441</v>
@@ -1782,16 +1809,16 @@
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A27" s="4" t="s">
-        <v>45</v>
+        <v>159</v>
       </c>
       <c r="B27" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C27" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D27" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="E27">
         <v>14</v>
@@ -1811,16 +1838,16 @@
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
-        <v>47</v>
+        <v>160</v>
       </c>
       <c r="B28" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="C28" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D28" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="E28">
         <v>14</v>
@@ -1843,13 +1870,13 @@
         <v>51</v>
       </c>
       <c r="B29" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="C29" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D29" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="E29">
         <v>14</v>
@@ -1869,16 +1896,16 @@
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A30" s="4" t="s">
-        <v>51</v>
+        <v>161</v>
       </c>
       <c r="B30" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="C30" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D30" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="E30">
         <v>14</v>
@@ -1901,13 +1928,13 @@
         <v>99</v>
       </c>
       <c r="B31" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="C31" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D31" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="E31">
         <v>14</v>
@@ -1930,13 +1957,13 @@
         <v>107</v>
       </c>
       <c r="B32" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="C32" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D32" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="E32">
         <v>14</v>
@@ -1959,13 +1986,13 @@
         <v>108</v>
       </c>
       <c r="B33" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="C33" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D33" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="E33">
         <v>14</v>
@@ -1988,13 +2015,13 @@
         <v>109</v>
       </c>
       <c r="B34" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="C34" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D34" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="E34">
         <v>14</v>
@@ -2017,13 +2044,13 @@
         <v>100</v>
       </c>
       <c r="B35" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="C35" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D35" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="E35">
         <v>14</v>
@@ -2046,13 +2073,13 @@
         <v>101</v>
       </c>
       <c r="B36" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="C36" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D36" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="E36">
         <v>14</v>
@@ -2075,13 +2102,13 @@
         <v>52</v>
       </c>
       <c r="B37" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="C37" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D37" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="E37">
         <v>14</v>
@@ -2104,13 +2131,13 @@
         <v>110</v>
       </c>
       <c r="B38" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="C38" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D38" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="E38">
         <v>14</v>
@@ -2130,16 +2157,16 @@
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A39" s="4" t="s">
-        <v>61</v>
+        <v>162</v>
       </c>
       <c r="B39" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="C39" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D39" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="E39">
         <v>14</v>
@@ -2162,13 +2189,13 @@
         <v>96</v>
       </c>
       <c r="B40" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="C40" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D40" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="E40">
         <v>14</v>
@@ -2188,16 +2215,16 @@
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A41" s="4" t="s">
-        <v>64</v>
+        <v>163</v>
       </c>
       <c r="B41" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="C41" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D41" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="E41">
         <v>14</v>
@@ -2217,16 +2244,16 @@
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A42" s="4" t="s">
-        <v>66</v>
+        <v>164</v>
       </c>
       <c r="B42" t="s">
-        <v>65</v>
+        <v>57</v>
       </c>
       <c r="C42" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D42" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="E42">
         <v>14</v>
@@ -2249,13 +2276,13 @@
         <v>46</v>
       </c>
       <c r="B43" t="s">
-        <v>67</v>
+        <v>58</v>
       </c>
       <c r="C43" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D43" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="E43">
         <v>14</v>
@@ -2278,13 +2305,13 @@
         <v>47</v>
       </c>
       <c r="B44" t="s">
-        <v>68</v>
+        <v>59</v>
       </c>
       <c r="C44" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D44" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="E44">
         <v>14</v>
@@ -2307,13 +2334,13 @@
         <v>102</v>
       </c>
       <c r="B45" t="s">
-        <v>69</v>
+        <v>60</v>
       </c>
       <c r="C45" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D45" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="E45">
         <v>14</v>
@@ -2332,23 +2359,23 @@
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A46" s="4" t="s">
-        <v>73</v>
+      <c r="A46" s="4">
+        <v>53</v>
       </c>
       <c r="B46" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="C46" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D46" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="E46">
         <v>14</v>
       </c>
       <c r="G46" s="5" t="s">
-        <v>71</v>
+        <v>62</v>
       </c>
       <c r="H46">
         <v>0</v>
@@ -2357,7 +2384,7 @@
         <v>0</v>
       </c>
       <c r="J46" s="6" t="s">
-        <v>72</v>
+        <v>63</v>
       </c>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.3">
@@ -2365,13 +2392,13 @@
         <v>54</v>
       </c>
       <c r="B47" t="s">
-        <v>74</v>
+        <v>64</v>
       </c>
       <c r="C47" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D47" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="E47">
         <v>14</v>
@@ -2394,13 +2421,13 @@
         <v>55</v>
       </c>
       <c r="B48" t="s">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="C48" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D48" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="E48">
         <v>14</v>
@@ -2423,13 +2450,13 @@
         <v>56</v>
       </c>
       <c r="B49" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="C49" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D49" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="E49">
         <v>14</v>
@@ -2452,13 +2479,13 @@
         <v>57</v>
       </c>
       <c r="B50" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="C50" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D50" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="E50">
         <v>14</v>
@@ -2477,17 +2504,17 @@
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A51">
-        <v>58</v>
+      <c r="A51" t="s">
+        <v>165</v>
       </c>
       <c r="B51" t="s">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="C51" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D51" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="E51">
         <v>14</v>
@@ -2510,13 +2537,13 @@
         <v>59</v>
       </c>
       <c r="B52" t="s">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="C52" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D52" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="E52">
         <v>14</v>
@@ -2539,13 +2566,13 @@
         <v>60</v>
       </c>
       <c r="B53" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="C53" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D53" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="E53">
         <v>14</v>
@@ -2568,13 +2595,13 @@
         <v>61</v>
       </c>
       <c r="B54" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="C54" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D54" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="E54">
         <v>14</v>
@@ -2597,13 +2624,13 @@
         <v>103</v>
       </c>
       <c r="B55" t="s">
-        <v>82</v>
+        <v>72</v>
       </c>
       <c r="C55" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D55" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="E55">
         <v>14</v>
@@ -2626,13 +2653,13 @@
         <v>104</v>
       </c>
       <c r="B56" t="s">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="C56" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D56" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="E56">
         <v>14</v>
@@ -2655,13 +2682,13 @@
         <v>105</v>
       </c>
       <c r="B57" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="C57" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D57" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="E57">
         <v>14</v>
@@ -2684,13 +2711,13 @@
         <v>106</v>
       </c>
       <c r="B58" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="C58" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D58" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="E58">
         <v>14</v>
@@ -2713,13 +2740,13 @@
         <v>97</v>
       </c>
       <c r="B59" t="s">
-        <v>86</v>
+        <v>76</v>
       </c>
       <c r="C59" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D59" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="E59">
         <v>14</v>
@@ -2742,13 +2769,13 @@
         <v>42</v>
       </c>
       <c r="B60" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="C60" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D60" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="E60">
         <v>14</v>
@@ -2768,16 +2795,16 @@
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A61" s="4" t="s">
-        <v>89</v>
+        <v>166</v>
       </c>
       <c r="B61" t="s">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="C61" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D61" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="E61">
         <v>15</v>
@@ -2800,13 +2827,13 @@
         <v>118</v>
       </c>
       <c r="B62" t="s">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="C62" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D62" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="E62">
         <v>15</v>
@@ -2829,13 +2856,13 @@
         <v>119</v>
       </c>
       <c r="B63" t="s">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="C63" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D63" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="E63">
         <v>15</v>
@@ -2858,13 +2885,13 @@
         <v>120</v>
       </c>
       <c r="B64" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="C64" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D64" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="E64">
         <v>15</v>
@@ -2887,13 +2914,13 @@
         <v>121</v>
       </c>
       <c r="B65" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="C65" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D65" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="E65">
         <v>15</v>
@@ -2916,13 +2943,13 @@
         <v>122</v>
       </c>
       <c r="B66" t="s">
-        <v>94</v>
+        <v>83</v>
       </c>
       <c r="C66" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D66" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="E66">
         <v>15</v>
@@ -2931,7 +2958,7 @@
         <v>46162.022916666669</v>
       </c>
       <c r="G66" s="6" t="s">
-        <v>95</v>
+        <v>84</v>
       </c>
       <c r="H66">
         <v>32</v>
@@ -2940,7 +2967,7 @@
         <v>0</v>
       </c>
       <c r="J66" s="6" t="s">
-        <v>96</v>
+        <v>85</v>
       </c>
     </row>
     <row r="67" spans="1:10" x14ac:dyDescent="0.3">
@@ -2948,13 +2975,13 @@
         <v>123</v>
       </c>
       <c r="B67" t="s">
-        <v>97</v>
+        <v>86</v>
       </c>
       <c r="C67" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D67" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="E67">
         <v>15</v>
@@ -2974,16 +3001,16 @@
     </row>
     <row r="68" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A68" s="4" t="s">
-        <v>99</v>
+        <v>167</v>
       </c>
       <c r="B68" t="s">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="C68" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D68" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="E68">
         <v>3</v>
@@ -3003,16 +3030,16 @@
     </row>
     <row r="69" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A69" s="4" t="s">
-        <v>102</v>
+        <v>168</v>
       </c>
       <c r="B69" t="s">
-        <v>100</v>
+        <v>88</v>
       </c>
       <c r="C69" t="s">
-        <v>101</v>
+        <v>89</v>
       </c>
       <c r="D69" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E69">
         <v>14</v>
@@ -3021,7 +3048,7 @@
         <v>46147.338888888888</v>
       </c>
       <c r="G69" s="6" t="s">
-        <v>95</v>
+        <v>84</v>
       </c>
       <c r="H69">
         <v>278</v>
@@ -3030,7 +3057,7 @@
         <v>0</v>
       </c>
       <c r="J69" s="6" t="s">
-        <v>96</v>
+        <v>85</v>
       </c>
     </row>
     <row r="70" spans="1:10" x14ac:dyDescent="0.3">
@@ -3038,13 +3065,13 @@
         <v>63</v>
       </c>
       <c r="B70" t="s">
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="C70" t="s">
-        <v>101</v>
+        <v>89</v>
       </c>
       <c r="D70" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E70">
         <v>14</v>
@@ -3063,17 +3090,17 @@
       </c>
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A71">
-        <v>64</v>
+      <c r="A71" t="s">
+        <v>169</v>
       </c>
       <c r="B71" t="s">
-        <v>104</v>
+        <v>91</v>
       </c>
       <c r="C71" t="s">
-        <v>101</v>
+        <v>89</v>
       </c>
       <c r="D71" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E71">
         <v>14</v>
@@ -3092,17 +3119,17 @@
       </c>
     </row>
     <row r="72" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A72">
-        <v>71</v>
+      <c r="A72" t="s">
+        <v>170</v>
       </c>
       <c r="B72" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="C72" t="s">
-        <v>101</v>
+        <v>89</v>
       </c>
       <c r="D72" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E72">
         <v>14</v>
@@ -3125,13 +3152,13 @@
         <v>66</v>
       </c>
       <c r="B73" t="s">
-        <v>106</v>
+        <v>93</v>
       </c>
       <c r="C73" t="s">
-        <v>101</v>
+        <v>89</v>
       </c>
       <c r="D73" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E73">
         <v>14</v>
@@ -3151,16 +3178,16 @@
     </row>
     <row r="74" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A74" s="4" t="s">
-        <v>108</v>
+        <v>171</v>
       </c>
       <c r="B74" t="s">
-        <v>107</v>
+        <v>94</v>
       </c>
       <c r="C74" t="s">
-        <v>101</v>
+        <v>89</v>
       </c>
       <c r="D74" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E74">
         <v>14</v>
@@ -3183,13 +3210,13 @@
         <v>68</v>
       </c>
       <c r="B75" t="s">
-        <v>109</v>
+        <v>95</v>
       </c>
       <c r="C75" t="s">
-        <v>101</v>
+        <v>89</v>
       </c>
       <c r="D75" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E75">
         <v>14</v>
@@ -3209,16 +3236,16 @@
     </row>
     <row r="76" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A76" s="4" t="s">
-        <v>111</v>
+        <v>172</v>
       </c>
       <c r="B76" t="s">
-        <v>110</v>
+        <v>96</v>
       </c>
       <c r="C76" t="s">
-        <v>101</v>
+        <v>89</v>
       </c>
       <c r="D76" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="E76">
         <v>14</v>
@@ -3227,7 +3254,7 @@
         <v>46162.020833333336</v>
       </c>
       <c r="G76" s="6" t="s">
-        <v>95</v>
+        <v>84</v>
       </c>
       <c r="H76">
         <v>15</v>
@@ -3236,7 +3263,7 @@
         <v>0</v>
       </c>
       <c r="J76" s="6" t="s">
-        <v>96</v>
+        <v>85</v>
       </c>
     </row>
     <row r="77" spans="1:10" x14ac:dyDescent="0.3">
@@ -3244,13 +3271,13 @@
         <v>115</v>
       </c>
       <c r="B77" t="s">
-        <v>112</v>
+        <v>97</v>
       </c>
       <c r="C77" t="s">
-        <v>101</v>
+        <v>89</v>
       </c>
       <c r="D77" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="E77">
         <v>14</v>
@@ -3273,13 +3300,13 @@
         <v>111</v>
       </c>
       <c r="B78" t="s">
-        <v>113</v>
+        <v>98</v>
       </c>
       <c r="C78" t="s">
-        <v>101</v>
+        <v>89</v>
       </c>
       <c r="D78" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="E78">
         <v>14</v>
@@ -3302,13 +3329,13 @@
         <v>112</v>
       </c>
       <c r="B79" t="s">
-        <v>114</v>
+        <v>99</v>
       </c>
       <c r="C79" t="s">
-        <v>101</v>
+        <v>89</v>
       </c>
       <c r="D79" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="E79">
         <v>14</v>
@@ -3331,13 +3358,13 @@
         <v>113</v>
       </c>
       <c r="B80" t="s">
-        <v>115</v>
+        <v>100</v>
       </c>
       <c r="C80" t="s">
-        <v>101</v>
+        <v>89</v>
       </c>
       <c r="D80" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="E80">
         <v>14</v>
@@ -3389,7 +3416,7 @@
   <sheetData>
     <row r="1" spans="1:20" ht="17.399999999999999" x14ac:dyDescent="0.35">
       <c r="A1" s="12" t="s">
-        <v>116</v>
+        <v>101</v>
       </c>
       <c r="B1" s="12"/>
       <c r="C1" s="12"/>
@@ -3413,7 +3440,7 @@
     </row>
     <row r="2" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A2" s="13" t="s">
-        <v>117</v>
+        <v>102</v>
       </c>
       <c r="B2" s="13"/>
       <c r="C2" s="13"/>
@@ -3461,45 +3488,45 @@
         <v>8</v>
       </c>
       <c r="I3" s="7" t="s">
-        <v>118</v>
+        <v>103</v>
       </c>
       <c r="J3" s="7" t="s">
-        <v>119</v>
+        <v>104</v>
       </c>
       <c r="K3" s="8" t="s">
-        <v>120</v>
+        <v>105</v>
       </c>
       <c r="L3" s="8" t="s">
-        <v>121</v>
+        <v>106</v>
       </c>
       <c r="M3" s="8" t="s">
-        <v>122</v>
+        <v>107</v>
       </c>
       <c r="N3" s="8" t="s">
-        <v>123</v>
+        <v>108</v>
       </c>
       <c r="O3" s="8" t="s">
-        <v>124</v>
+        <v>109</v>
       </c>
       <c r="P3" s="8" t="s">
-        <v>125</v>
+        <v>110</v>
       </c>
       <c r="Q3" s="8" t="s">
-        <v>126</v>
+        <v>111</v>
       </c>
       <c r="R3" s="8" t="s">
-        <v>127</v>
+        <v>112</v>
       </c>
       <c r="S3" s="8" t="s">
-        <v>128</v>
+        <v>113</v>
       </c>
       <c r="T3" s="8" t="s">
-        <v>129</v>
+        <v>114</v>
       </c>
     </row>
     <row r="4" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A4" s="10" t="s">
-        <v>130</v>
+        <v>115</v>
       </c>
       <c r="B4" s="10" t="s">
         <v>11</v>
@@ -3524,7 +3551,7 @@
       </c>
       <c r="I4" s="10"/>
       <c r="J4" s="10" t="s">
-        <v>131</v>
+        <v>116</v>
       </c>
       <c r="K4" s="9">
         <v>4</v>
@@ -3557,13 +3584,13 @@
     </row>
     <row r="5" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>132</v>
+        <v>117</v>
       </c>
       <c r="B5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D5">
         <v>14</v>
@@ -3581,7 +3608,7 @@
         <v>0</v>
       </c>
       <c r="J5" t="s">
-        <v>131</v>
+        <v>116</v>
       </c>
       <c r="K5" s="9">
         <v>3</v>
@@ -3612,18 +3639,18 @@
         <v>3.5</v>
       </c>
       <c r="T5" t="s">
-        <v>160</v>
+        <v>145</v>
       </c>
     </row>
     <row r="6" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A6" s="10" t="s">
-        <v>133</v>
+        <v>118</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D6" s="10">
         <v>14</v>
@@ -3642,7 +3669,7 @@
       </c>
       <c r="I6" s="10"/>
       <c r="J6" s="10" t="s">
-        <v>131</v>
+        <v>116</v>
       </c>
       <c r="K6" s="9"/>
       <c r="L6" s="9"/>
@@ -3659,13 +3686,13 @@
     </row>
     <row r="7" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>134</v>
+        <v>119</v>
       </c>
       <c r="B7" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C7" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="D7">
         <v>14</v>
@@ -3683,7 +3710,7 @@
         <v>0</v>
       </c>
       <c r="J7" t="s">
-        <v>131</v>
+        <v>116</v>
       </c>
       <c r="K7" s="9"/>
       <c r="L7" s="9"/>
@@ -3700,13 +3727,13 @@
     </row>
     <row r="8" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A8" s="10" t="s">
-        <v>135</v>
+        <v>120</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="D8" s="10">
         <v>14</v>
@@ -3725,7 +3752,7 @@
       </c>
       <c r="I8" s="10"/>
       <c r="J8" s="10" t="s">
-        <v>131</v>
+        <v>116</v>
       </c>
       <c r="K8" s="9"/>
       <c r="L8" s="9"/>
@@ -3742,13 +3769,13 @@
     </row>
     <row r="9" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>136</v>
+        <v>121</v>
       </c>
       <c r="B9" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C9" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="D9">
         <v>14</v>
@@ -3766,7 +3793,7 @@
         <v>0</v>
       </c>
       <c r="J9" t="s">
-        <v>131</v>
+        <v>116</v>
       </c>
       <c r="K9" s="9"/>
       <c r="L9" s="9"/>
@@ -3783,13 +3810,13 @@
     </row>
     <row r="10" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A10" s="10" t="s">
-        <v>137</v>
+        <v>122</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="D10" s="10">
         <v>14</v>
@@ -3808,7 +3835,7 @@
       </c>
       <c r="I10" s="10"/>
       <c r="J10" s="10" t="s">
-        <v>131</v>
+        <v>116</v>
       </c>
       <c r="K10" s="9">
         <v>4</v>
@@ -3841,13 +3868,13 @@
     </row>
     <row r="11" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>163</v>
+        <v>148</v>
       </c>
       <c r="B11" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C11" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="D11">
         <v>14</v>
@@ -3866,7 +3893,7 @@
       </c>
       <c r="I11" s="6"/>
       <c r="J11" t="s">
-        <v>131</v>
+        <v>116</v>
       </c>
       <c r="K11" s="9"/>
       <c r="L11" s="9"/>
@@ -3879,13 +3906,13 @@
     </row>
     <row r="12" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A12" s="10" t="s">
-        <v>138</v>
+        <v>123</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="D12" s="10">
         <v>14</v>
@@ -3904,7 +3931,7 @@
       </c>
       <c r="I12" s="10"/>
       <c r="J12" s="10" t="s">
-        <v>131</v>
+        <v>116</v>
       </c>
       <c r="K12" s="9"/>
       <c r="L12" s="9"/>
@@ -3921,13 +3948,13 @@
     </row>
     <row r="13" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>139</v>
+        <v>124</v>
       </c>
       <c r="B13" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C13" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="D13">
         <v>14</v>
@@ -3945,7 +3972,7 @@
         <v>0</v>
       </c>
       <c r="J13" t="s">
-        <v>131</v>
+        <v>116</v>
       </c>
       <c r="K13" s="9"/>
       <c r="L13" s="9"/>
@@ -3962,13 +3989,13 @@
     </row>
     <row r="14" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A14" s="10" t="s">
-        <v>140</v>
+        <v>125</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="D14" s="10">
         <v>15</v>
@@ -3987,7 +4014,7 @@
       </c>
       <c r="I14" s="10"/>
       <c r="J14" s="10" t="s">
-        <v>131</v>
+        <v>116</v>
       </c>
       <c r="K14" s="9"/>
       <c r="L14" s="9"/>
@@ -4004,13 +4031,13 @@
     </row>
     <row r="15" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>141</v>
+        <v>126</v>
       </c>
       <c r="B15" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C15" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="D15">
         <v>3</v>
@@ -4028,7 +4055,7 @@
         <v>0</v>
       </c>
       <c r="J15" t="s">
-        <v>131</v>
+        <v>116</v>
       </c>
       <c r="K15" s="9"/>
       <c r="L15" s="9"/>
@@ -4045,13 +4072,13 @@
     </row>
     <row r="16" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A16" s="10" t="s">
-        <v>142</v>
+        <v>127</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>101</v>
+        <v>89</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D16" s="10">
         <v>14</v>
@@ -4060,7 +4087,7 @@
         <v>46147.338888888888</v>
       </c>
       <c r="F16" s="10" t="s">
-        <v>95</v>
+        <v>84</v>
       </c>
       <c r="G16" s="10">
         <v>278</v>
@@ -4069,10 +4096,10 @@
         <v>0</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>143</v>
+        <v>128</v>
       </c>
       <c r="J16" s="10" t="s">
-        <v>131</v>
+        <v>116</v>
       </c>
       <c r="K16" s="9">
         <v>5</v>
@@ -4105,13 +4132,13 @@
     </row>
     <row r="17" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>144</v>
+        <v>129</v>
       </c>
       <c r="B17" t="s">
-        <v>101</v>
+        <v>89</v>
       </c>
       <c r="C17" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D17">
         <v>14</v>
@@ -4129,7 +4156,7 @@
         <v>0</v>
       </c>
       <c r="J17" t="s">
-        <v>131</v>
+        <v>116</v>
       </c>
       <c r="K17" s="9">
         <v>3</v>
@@ -4160,18 +4187,18 @@
         <v>3.5</v>
       </c>
       <c r="T17" t="s">
-        <v>162</v>
+        <v>147</v>
       </c>
     </row>
     <row r="18" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A18" s="10" t="s">
-        <v>145</v>
+        <v>130</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>101</v>
+        <v>89</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="D18" s="10">
         <v>14</v>
@@ -4180,7 +4207,7 @@
         <v>46162.020833333336</v>
       </c>
       <c r="F18" s="10" t="s">
-        <v>95</v>
+        <v>84</v>
       </c>
       <c r="G18" s="10">
         <v>15</v>
@@ -4189,10 +4216,10 @@
         <v>0</v>
       </c>
       <c r="I18" s="10" t="s">
-        <v>143</v>
+        <v>128</v>
       </c>
       <c r="J18" s="10" t="s">
-        <v>131</v>
+        <v>116</v>
       </c>
       <c r="K18" s="9">
         <v>5</v>
@@ -4225,7 +4252,7 @@
     </row>
     <row r="20" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A20" s="10" t="s">
-        <v>147</v>
+        <v>132</v>
       </c>
       <c r="B20" s="10" t="s">
         <v>11</v>
@@ -4250,7 +4277,7 @@
       </c>
       <c r="I20" s="10"/>
       <c r="J20" s="10" t="s">
-        <v>131</v>
+        <v>116</v>
       </c>
       <c r="K20" s="9">
         <v>3</v>
@@ -4281,12 +4308,12 @@
         <v>3.375</v>
       </c>
       <c r="T20" t="s">
-        <v>156</v>
+        <v>141</v>
       </c>
     </row>
     <row r="21" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>148</v>
+        <v>133</v>
       </c>
       <c r="B21" t="s">
         <v>11</v>
@@ -4310,7 +4337,7 @@
         <v>0</v>
       </c>
       <c r="J21" t="s">
-        <v>131</v>
+        <v>116</v>
       </c>
       <c r="K21" s="9">
         <v>3</v>
@@ -4343,13 +4370,13 @@
     </row>
     <row r="22" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A22" s="10" t="s">
-        <v>149</v>
+        <v>134</v>
       </c>
       <c r="B22" s="10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C22" s="10" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D22" s="10">
         <v>14</v>
@@ -4368,7 +4395,7 @@
       </c>
       <c r="I22" s="10"/>
       <c r="J22" s="10" t="s">
-        <v>131</v>
+        <v>116</v>
       </c>
       <c r="K22" s="9">
         <v>2</v>
@@ -4399,18 +4426,18 @@
         <v>3.375</v>
       </c>
       <c r="T22" t="s">
-        <v>161</v>
+        <v>146</v>
       </c>
     </row>
     <row r="23" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>150</v>
+        <v>135</v>
       </c>
       <c r="B23" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C23" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D23">
         <v>14</v>
@@ -4428,7 +4455,7 @@
         <v>0</v>
       </c>
       <c r="J23" t="s">
-        <v>131</v>
+        <v>116</v>
       </c>
       <c r="K23" s="9">
         <v>4</v>
@@ -4459,18 +4486,18 @@
         <v>3.25</v>
       </c>
       <c r="T23" t="s">
-        <v>159</v>
+        <v>144</v>
       </c>
     </row>
     <row r="24" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A24" s="10" t="s">
-        <v>151</v>
+        <v>136</v>
       </c>
       <c r="B24" s="10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C24" s="10" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D24" s="10">
         <v>14</v>
@@ -4489,7 +4516,7 @@
       </c>
       <c r="I24" s="10"/>
       <c r="J24" s="10" t="s">
-        <v>131</v>
+        <v>116</v>
       </c>
       <c r="K24" s="9">
         <v>4</v>
@@ -4522,13 +4549,13 @@
     </row>
     <row r="25" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>152</v>
+        <v>137</v>
       </c>
       <c r="B25" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C25" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D25">
         <v>14</v>
@@ -4546,7 +4573,7 @@
         <v>0</v>
       </c>
       <c r="J25" t="s">
-        <v>131</v>
+        <v>116</v>
       </c>
       <c r="K25" s="9"/>
       <c r="L25" s="9"/>
@@ -4563,13 +4590,13 @@
     </row>
     <row r="26" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A26" s="10" t="s">
-        <v>153</v>
+        <v>138</v>
       </c>
       <c r="B26" s="10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C26" s="10" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D26" s="10">
         <v>14</v>
@@ -4588,7 +4615,7 @@
       </c>
       <c r="I26" s="10"/>
       <c r="J26" s="10" t="s">
-        <v>131</v>
+        <v>116</v>
       </c>
       <c r="K26" s="9">
         <v>3</v>
@@ -4621,13 +4648,13 @@
     </row>
     <row r="27" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>154</v>
+        <v>139</v>
       </c>
       <c r="B27" t="s">
-        <v>101</v>
+        <v>89</v>
       </c>
       <c r="C27" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D27">
         <v>14</v>
@@ -4645,7 +4672,7 @@
         <v>0</v>
       </c>
       <c r="J27" t="s">
-        <v>131</v>
+        <v>116</v>
       </c>
       <c r="K27" s="9">
         <v>3</v>
@@ -4676,18 +4703,18 @@
         <v>3.375</v>
       </c>
       <c r="T27" t="s">
-        <v>158</v>
+        <v>143</v>
       </c>
     </row>
     <row r="28" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A28" s="10" t="s">
-        <v>155</v>
+        <v>140</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>101</v>
+        <v>89</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D28" s="10">
         <v>14</v>
@@ -4706,7 +4733,7 @@
       </c>
       <c r="I28" s="10"/>
       <c r="J28" s="10" t="s">
-        <v>131</v>
+        <v>116</v>
       </c>
       <c r="K28" s="9">
         <v>4</v>
@@ -4737,12 +4764,12 @@
         <v>3.375</v>
       </c>
       <c r="T28" t="s">
-        <v>157</v>
+        <v>142</v>
       </c>
     </row>
     <row r="29" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A29" s="14" t="s">
-        <v>146</v>
+        <v>131</v>
       </c>
       <c r="B29" s="14"/>
       <c r="C29" s="14"/>

</xml_diff>

<commit_message>
Checklist: clear sample highlight from TN Custom Media (ID 53, row 46)
</commit_message>
<xml_diff>
--- a/doc_readiness_checklist.xlsx
+++ b/doc_readiness_checklist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\AQCWT\OpenCode_Doc\APAI_Chat\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF931B3E-1FA1-4C33-8D21-500D2F26ED9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32B33CFD-7388-4A0B-B878-C14836EB812C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{BE8B64C7-7DD3-42E9-8432-DA4C4DC91B80}"/>
   </bookViews>
@@ -614,7 +614,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -675,6 +675,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -688,7 +694,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -704,6 +710,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2359,7 +2366,7 @@
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A46" s="4">
+      <c r="A46" s="15">
         <v>53</v>
       </c>
       <c r="B46" t="s">

</xml_diff>

<commit_message>
Checklist: add ID column to Readiness Checklist sheet for cross-reference
</commit_message>
<xml_diff>
--- a/doc_readiness_checklist.xlsx
+++ b/doc_readiness_checklist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\AQCWT\OpenCode_Doc\APAI_Chat\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32B33CFD-7388-4A0B-B878-C14836EB812C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D6C8872-1C76-4250-947E-B2D01FB77EA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{BE8B64C7-7DD3-42E9-8432-DA4C4DC91B80}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="506" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="507" uniqueCount="173">
   <si>
     <t>ID</t>
   </si>
@@ -694,7 +694,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -707,10 +707,11 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="22" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2366,7 +2367,7 @@
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A46" s="15">
+      <c r="A46" s="12">
         <v>53</v>
       </c>
       <c r="B46" t="s">
@@ -3396,173 +3397,177 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{299327EC-E1E5-4A36-9AAD-A1F4644DF0C0}">
-  <dimension ref="A1:T29"/>
+  <dimension ref="A1:U29"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="80.77734375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.77734375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.21875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="20.6640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="7.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.5546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18.88671875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="17.33203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="17.77734375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="16.109375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="17.77734375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="16.88671875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="17.5546875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="15.33203125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="19.21875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="9" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="12.77734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.77734375" customWidth="1"/>
+    <col min="2" max="2" width="80.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="7.21875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="7.109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.5546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="18.88671875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="17.77734375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="17.77734375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="16.88671875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="17.5546875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="19.21875" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="9" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="12.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" ht="17.399999999999999" x14ac:dyDescent="0.35">
-      <c r="A1" s="12" t="s">
+    <row r="1" spans="1:21" ht="17.399999999999999" x14ac:dyDescent="0.35">
+      <c r="B1" s="13" t="s">
         <v>101</v>
       </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
-      <c r="H1" s="12"/>
-      <c r="I1" s="12"/>
-      <c r="J1" s="12"/>
-      <c r="K1" s="12"/>
-      <c r="L1" s="12"/>
-      <c r="M1" s="12"/>
-      <c r="N1" s="12"/>
-      <c r="O1" s="12"/>
-      <c r="P1" s="12"/>
-      <c r="Q1" s="12"/>
-      <c r="R1" s="12"/>
-      <c r="S1" s="12"/>
-      <c r="T1" s="12"/>
-    </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A2" s="13" t="s">
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13"/>
+      <c r="I1" s="13"/>
+      <c r="J1" s="13"/>
+      <c r="K1" s="13"/>
+      <c r="L1" s="13"/>
+      <c r="M1" s="13"/>
+      <c r="N1" s="13"/>
+      <c r="O1" s="13"/>
+      <c r="P1" s="13"/>
+      <c r="Q1" s="13"/>
+      <c r="R1" s="13"/>
+      <c r="S1" s="13"/>
+      <c r="T1" s="13"/>
+      <c r="U1" s="13"/>
+    </row>
+    <row r="2" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="B2" s="14" t="s">
         <v>102</v>
       </c>
-      <c r="B2" s="13"/>
-      <c r="C2" s="13"/>
-      <c r="D2" s="13"/>
-      <c r="E2" s="13"/>
-      <c r="F2" s="13"/>
-      <c r="G2" s="13"/>
-      <c r="H2" s="13"/>
-      <c r="I2" s="13"/>
-      <c r="J2" s="13"/>
-      <c r="K2" s="13"/>
-      <c r="L2" s="13"/>
-      <c r="M2" s="13"/>
-      <c r="N2" s="13"/>
-      <c r="O2" s="13"/>
-      <c r="P2" s="13"/>
-      <c r="Q2" s="13"/>
-      <c r="R2" s="13"/>
-      <c r="S2" s="13"/>
-      <c r="T2" s="13"/>
-    </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
+      <c r="H2" s="14"/>
+      <c r="I2" s="14"/>
+      <c r="J2" s="14"/>
+      <c r="K2" s="14"/>
+      <c r="L2" s="14"/>
+      <c r="M2" s="14"/>
+      <c r="N2" s="14"/>
+      <c r="O2" s="14"/>
+      <c r="P2" s="14"/>
+      <c r="Q2" s="14"/>
+      <c r="R2" s="14"/>
+      <c r="S2" s="14"/>
+      <c r="T2" s="14"/>
+      <c r="U2" s="14"/>
+    </row>
+    <row r="3" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A3" s="16" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="C3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="D3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="1" t="s">
-        <v>4</v>
-      </c>
       <c r="E3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F3" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="G3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="H3" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="H3" s="7" t="s">
+      <c r="I3" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="I3" s="7" t="s">
+      <c r="J3" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="J3" s="7" t="s">
+      <c r="K3" s="7" t="s">
         <v>104</v>
       </c>
-      <c r="K3" s="8" t="s">
+      <c r="L3" s="8" t="s">
         <v>105</v>
       </c>
-      <c r="L3" s="8" t="s">
+      <c r="M3" s="8" t="s">
         <v>106</v>
       </c>
-      <c r="M3" s="8" t="s">
+      <c r="N3" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="N3" s="8" t="s">
+      <c r="O3" s="8" t="s">
         <v>108</v>
       </c>
-      <c r="O3" s="8" t="s">
+      <c r="P3" s="8" t="s">
         <v>109</v>
       </c>
-      <c r="P3" s="8" t="s">
+      <c r="Q3" s="8" t="s">
         <v>110</v>
       </c>
-      <c r="Q3" s="8" t="s">
+      <c r="R3" s="8" t="s">
         <v>111</v>
       </c>
-      <c r="R3" s="8" t="s">
+      <c r="S3" s="8" t="s">
         <v>112</v>
       </c>
-      <c r="S3" s="8" t="s">
+      <c r="T3" s="8" t="s">
         <v>113</v>
       </c>
-      <c r="T3" s="8" t="s">
+      <c r="U3" s="8" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A4" s="10" t="s">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>124</v>
+      </c>
+      <c r="B4" s="10" t="s">
         <v>115</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="C4" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="D4" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="10">
-        <v>14</v>
-      </c>
-      <c r="E4" s="11">
+      <c r="E4" s="10">
+        <v>14</v>
+      </c>
+      <c r="F4" s="11">
         <v>46175.950694444444</v>
       </c>
-      <c r="F4" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="G4" s="10">
+      <c r="G4" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="H4" s="10">
         <v>2</v>
       </c>
-      <c r="H4" s="10">
-        <v>0</v>
-      </c>
-      <c r="I4" s="10"/>
-      <c r="J4" s="10" t="s">
+      <c r="I4" s="10">
+        <v>0</v>
+      </c>
+      <c r="J4" s="10"/>
+      <c r="K4" s="10" t="s">
         <v>116</v>
       </c>
-      <c r="K4" s="9">
-        <v>4</v>
-      </c>
       <c r="L4" s="9">
         <v>4</v>
       </c>
@@ -3573,56 +3578,59 @@
         <v>4</v>
       </c>
       <c r="O4" s="9">
+        <v>4</v>
+      </c>
+      <c r="P4" s="9">
         <v>3</v>
       </c>
-      <c r="P4" s="9">
-        <v>4</v>
-      </c>
       <c r="Q4" s="9">
+        <v>4</v>
+      </c>
+      <c r="R4" s="9">
         <v>3</v>
       </c>
-      <c r="R4" s="9">
-        <v>4</v>
-      </c>
-      <c r="S4">
-        <f t="shared" ref="S4:S18" si="0">IFERROR(AVERAGE(K4:R4),"")</f>
+      <c r="S4" s="9">
+        <v>4</v>
+      </c>
+      <c r="T4">
+        <f t="shared" ref="T4:T18" si="0">IFERROR(AVERAGE(L4:S4),"")</f>
         <v>3.75</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>76</v>
+      </c>
+      <c r="B5" t="s">
         <v>117</v>
       </c>
-      <c r="B5" t="s">
-        <v>20</v>
-      </c>
       <c r="C5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D5" t="s">
         <v>18</v>
       </c>
-      <c r="D5">
-        <v>14</v>
-      </c>
-      <c r="E5" s="2">
+      <c r="E5">
+        <v>14</v>
+      </c>
+      <c r="F5" s="2">
         <v>46161.998611111114</v>
       </c>
-      <c r="F5" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="G5">
+      <c r="G5" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="H5">
         <v>1</v>
       </c>
-      <c r="H5">
-        <v>0</v>
-      </c>
-      <c r="J5" t="s">
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="K5" t="s">
         <v>116</v>
       </c>
-      <c r="K5" s="9">
+      <c r="L5" s="9">
         <v>3</v>
       </c>
-      <c r="L5" s="9">
-        <v>4</v>
-      </c>
       <c r="M5" s="9">
         <v>4</v>
       </c>
@@ -3630,55 +3638,60 @@
         <v>4</v>
       </c>
       <c r="O5" s="9">
+        <v>4</v>
+      </c>
+      <c r="P5" s="9">
         <v>5</v>
-      </c>
-      <c r="P5" s="9">
-        <v>2</v>
       </c>
       <c r="Q5" s="9">
         <v>2</v>
       </c>
       <c r="R5" s="9">
-        <v>4</v>
-      </c>
-      <c r="S5">
+        <v>2</v>
+      </c>
+      <c r="S5" s="9">
+        <v>4</v>
+      </c>
+      <c r="T5">
         <f t="shared" si="0"/>
         <v>3.5</v>
       </c>
-      <c r="T5" t="s">
+      <c r="U5" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A6" s="10" t="s">
+    <row r="6" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>39</v>
+      </c>
+      <c r="B6" s="10" t="s">
         <v>118</v>
       </c>
-      <c r="B6" s="10" t="s">
-        <v>20</v>
-      </c>
       <c r="C6" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="D6" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="D6" s="10">
-        <v>14</v>
-      </c>
-      <c r="E6" s="11">
+      <c r="E6" s="10">
+        <v>14</v>
+      </c>
+      <c r="F6" s="11">
         <v>46147.351388888892</v>
       </c>
-      <c r="F6" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="G6" s="10">
+      <c r="G6" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="H6" s="10">
         <v>1342</v>
       </c>
-      <c r="H6" s="10">
-        <v>0</v>
-      </c>
-      <c r="I6" s="10"/>
-      <c r="J6" s="10" t="s">
+      <c r="I6" s="10">
+        <v>0</v>
+      </c>
+      <c r="J6" s="10"/>
+      <c r="K6" s="10" t="s">
         <v>116</v>
       </c>
-      <c r="K6" s="9"/>
       <c r="L6" s="9"/>
       <c r="M6" s="9"/>
       <c r="N6" s="9"/>
@@ -3686,40 +3699,43 @@
       <c r="P6" s="9"/>
       <c r="Q6" s="9"/>
       <c r="R6" s="9"/>
-      <c r="S6" t="str">
+      <c r="S6" s="9"/>
+      <c r="T6" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
+    <row r="7" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>62</v>
+      </c>
+      <c r="B7" t="s">
         <v>119</v>
       </c>
-      <c r="B7" t="s">
-        <v>20</v>
-      </c>
       <c r="C7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7" t="s">
         <v>40</v>
       </c>
-      <c r="D7">
-        <v>14</v>
-      </c>
-      <c r="E7" s="2">
+      <c r="E7">
+        <v>14</v>
+      </c>
+      <c r="F7" s="2">
         <v>46153.372916666667</v>
       </c>
-      <c r="F7" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="G7">
+      <c r="G7" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="H7">
         <v>320</v>
       </c>
-      <c r="H7">
-        <v>0</v>
-      </c>
-      <c r="J7" t="s">
+      <c r="I7">
+        <v>0</v>
+      </c>
+      <c r="K7" t="s">
         <v>116</v>
       </c>
-      <c r="K7" s="9"/>
       <c r="L7" s="9"/>
       <c r="M7" s="9"/>
       <c r="N7" s="9"/>
@@ -3727,41 +3743,44 @@
       <c r="P7" s="9"/>
       <c r="Q7" s="9"/>
       <c r="R7" s="9"/>
-      <c r="S7" t="str">
+      <c r="S7" s="9"/>
+      <c r="T7" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A8" s="10" t="s">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>43</v>
+      </c>
+      <c r="B8" s="10" t="s">
         <v>120</v>
       </c>
-      <c r="B8" s="10" t="s">
-        <v>20</v>
-      </c>
       <c r="C8" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="D8" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="D8" s="10">
-        <v>14</v>
-      </c>
-      <c r="E8" s="11">
+      <c r="E8" s="10">
+        <v>14</v>
+      </c>
+      <c r="F8" s="11">
         <v>46149.958333333336</v>
       </c>
-      <c r="F8" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="G8" s="10">
+      <c r="G8" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="H8" s="10">
         <v>142</v>
       </c>
-      <c r="H8" s="10">
-        <v>0</v>
-      </c>
-      <c r="I8" s="10"/>
-      <c r="J8" s="10" t="s">
+      <c r="I8" s="10">
+        <v>0</v>
+      </c>
+      <c r="J8" s="10"/>
+      <c r="K8" s="10" t="s">
         <v>116</v>
       </c>
-      <c r="K8" s="9"/>
       <c r="L8" s="9"/>
       <c r="M8" s="9"/>
       <c r="N8" s="9"/>
@@ -3769,40 +3788,43 @@
       <c r="P8" s="9"/>
       <c r="Q8" s="9"/>
       <c r="R8" s="9"/>
-      <c r="S8" t="str">
+      <c r="S8" s="9"/>
+      <c r="T8" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
+    <row r="9" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>98</v>
+      </c>
+      <c r="B9" t="s">
         <v>121</v>
       </c>
-      <c r="B9" t="s">
-        <v>20</v>
-      </c>
       <c r="C9" t="s">
-        <v>44</v>
-      </c>
-      <c r="D9">
-        <v>14</v>
-      </c>
-      <c r="E9" s="2">
+        <v>20</v>
+      </c>
+      <c r="D9" t="s">
+        <v>44</v>
+      </c>
+      <c r="E9">
+        <v>14</v>
+      </c>
+      <c r="F9" s="2">
         <v>46162.01666666667</v>
       </c>
-      <c r="F9" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="G9">
+      <c r="G9" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="H9">
         <v>15</v>
       </c>
-      <c r="H9">
-        <v>0</v>
-      </c>
-      <c r="J9" t="s">
+      <c r="I9">
+        <v>0</v>
+      </c>
+      <c r="K9" t="s">
         <v>116</v>
       </c>
-      <c r="K9" s="9"/>
       <c r="L9" s="9"/>
       <c r="M9" s="9"/>
       <c r="N9" s="9"/>
@@ -3810,99 +3832,105 @@
       <c r="P9" s="9"/>
       <c r="Q9" s="9"/>
       <c r="R9" s="9"/>
-      <c r="S9" t="str">
+      <c r="S9" s="9"/>
+      <c r="T9" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A10" s="10" t="s">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>95</v>
+      </c>
+      <c r="B10" s="10" t="s">
         <v>122</v>
       </c>
-      <c r="B10" s="10" t="s">
-        <v>20</v>
-      </c>
       <c r="C10" s="10" t="s">
-        <v>44</v>
-      </c>
-      <c r="D10" s="10">
-        <v>14</v>
-      </c>
-      <c r="E10" s="11">
+        <v>20</v>
+      </c>
+      <c r="D10" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="E10" s="10">
+        <v>14</v>
+      </c>
+      <c r="F10" s="11">
         <v>46162.013194444444</v>
       </c>
-      <c r="F10" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="G10" s="10">
+      <c r="G10" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="H10" s="10">
         <v>12</v>
       </c>
-      <c r="H10" s="10">
-        <v>0</v>
-      </c>
-      <c r="I10" s="10"/>
-      <c r="J10" s="10" t="s">
+      <c r="I10" s="10">
+        <v>0</v>
+      </c>
+      <c r="J10" s="10"/>
+      <c r="K10" s="10" t="s">
         <v>116</v>
       </c>
-      <c r="K10" s="9">
-        <v>4</v>
-      </c>
       <c r="L10" s="9">
+        <v>4</v>
+      </c>
+      <c r="M10" s="9">
         <v>3</v>
       </c>
-      <c r="M10" s="9">
-        <v>4</v>
-      </c>
       <c r="N10" s="9">
+        <v>4</v>
+      </c>
+      <c r="O10" s="9">
         <v>5</v>
       </c>
-      <c r="O10" s="9">
+      <c r="P10" s="9">
         <v>3</v>
       </c>
-      <c r="P10" s="9">
+      <c r="Q10" s="9">
         <v>5</v>
-      </c>
-      <c r="Q10" s="9">
-        <v>3</v>
       </c>
       <c r="R10" s="9">
         <v>3</v>
       </c>
-      <c r="S10">
+      <c r="S10" s="9">
+        <v>3</v>
+      </c>
+      <c r="T10">
         <f t="shared" si="0"/>
         <v>3.75</v>
       </c>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
+    <row r="11" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>58</v>
+      </c>
+      <c r="B11" t="s">
         <v>148</v>
       </c>
-      <c r="B11" t="s">
-        <v>20</v>
-      </c>
       <c r="C11" t="s">
-        <v>44</v>
-      </c>
-      <c r="D11">
-        <v>14</v>
-      </c>
-      <c r="E11" s="2">
+        <v>20</v>
+      </c>
+      <c r="D11" t="s">
+        <v>44</v>
+      </c>
+      <c r="E11">
+        <v>14</v>
+      </c>
+      <c r="F11" s="2">
         <v>46150.365972222222</v>
       </c>
-      <c r="F11" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G11">
+      <c r="G11" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="H11">
         <v>22</v>
       </c>
-      <c r="H11">
-        <v>0</v>
-      </c>
-      <c r="I11" s="6"/>
-      <c r="J11" t="s">
+      <c r="I11">
+        <v>0</v>
+      </c>
+      <c r="J11" s="6"/>
+      <c r="K11" t="s">
         <v>116</v>
       </c>
-      <c r="K11" s="9"/>
       <c r="L11" s="9"/>
       <c r="M11" s="9"/>
       <c r="N11" s="9"/>
@@ -3910,37 +3938,40 @@
       <c r="P11" s="9"/>
       <c r="Q11" s="9"/>
       <c r="R11" s="9"/>
-    </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A12" s="10" t="s">
+      <c r="S11" s="9"/>
+    </row>
+    <row r="12" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A12">
+        <v>45</v>
+      </c>
+      <c r="B12" s="10" t="s">
         <v>123</v>
       </c>
-      <c r="B12" s="10" t="s">
-        <v>20</v>
-      </c>
       <c r="C12" s="10" t="s">
-        <v>44</v>
-      </c>
-      <c r="D12" s="10">
-        <v>14</v>
-      </c>
-      <c r="E12" s="11">
+        <v>20</v>
+      </c>
+      <c r="D12" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="E12" s="10">
+        <v>14</v>
+      </c>
+      <c r="F12" s="11">
         <v>46149.957638888889</v>
       </c>
-      <c r="F12" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="G12" s="10">
+      <c r="G12" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="H12" s="10">
         <v>16</v>
       </c>
-      <c r="H12" s="10">
-        <v>0</v>
-      </c>
-      <c r="I12" s="10"/>
-      <c r="J12" s="10" t="s">
+      <c r="I12" s="10">
+        <v>0</v>
+      </c>
+      <c r="J12" s="10"/>
+      <c r="K12" s="10" t="s">
         <v>116</v>
       </c>
-      <c r="K12" s="9"/>
       <c r="L12" s="9"/>
       <c r="M12" s="9"/>
       <c r="N12" s="9"/>
@@ -3948,40 +3979,43 @@
       <c r="P12" s="9"/>
       <c r="Q12" s="9"/>
       <c r="R12" s="9"/>
-      <c r="S12" t="str">
+      <c r="S12" s="9"/>
+      <c r="T12" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
+    <row r="13" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>44</v>
+      </c>
+      <c r="B13" t="s">
         <v>124</v>
       </c>
-      <c r="B13" t="s">
-        <v>20</v>
-      </c>
       <c r="C13" t="s">
-        <v>44</v>
-      </c>
-      <c r="D13">
-        <v>14</v>
-      </c>
-      <c r="E13" s="2">
+        <v>20</v>
+      </c>
+      <c r="D13" t="s">
+        <v>44</v>
+      </c>
+      <c r="E13">
+        <v>14</v>
+      </c>
+      <c r="F13" s="2">
         <v>46149.957638888889</v>
       </c>
-      <c r="F13" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="G13">
+      <c r="G13" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="H13">
         <v>19</v>
       </c>
-      <c r="H13">
-        <v>0</v>
-      </c>
-      <c r="J13" t="s">
+      <c r="I13">
+        <v>0</v>
+      </c>
+      <c r="K13" t="s">
         <v>116</v>
       </c>
-      <c r="K13" s="9"/>
       <c r="L13" s="9"/>
       <c r="M13" s="9"/>
       <c r="N13" s="9"/>
@@ -3989,41 +4023,44 @@
       <c r="P13" s="9"/>
       <c r="Q13" s="9"/>
       <c r="R13" s="9"/>
-      <c r="S13" t="str">
+      <c r="S13" s="9"/>
+      <c r="T13" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A14" s="10" t="s">
+    <row r="14" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>117</v>
+      </c>
+      <c r="B14" s="10" t="s">
         <v>125</v>
       </c>
-      <c r="B14" s="10" t="s">
-        <v>20</v>
-      </c>
       <c r="C14" s="10" t="s">
-        <v>44</v>
-      </c>
-      <c r="D14" s="10">
+        <v>20</v>
+      </c>
+      <c r="D14" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="E14" s="10">
         <v>15</v>
       </c>
-      <c r="E14" s="11">
+      <c r="F14" s="11">
         <v>46162.022916666669</v>
       </c>
-      <c r="F14" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="G14" s="10">
+      <c r="G14" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="H14" s="10">
         <v>21</v>
       </c>
-      <c r="H14" s="10">
-        <v>0</v>
-      </c>
-      <c r="I14" s="10"/>
-      <c r="J14" s="10" t="s">
+      <c r="I14" s="10">
+        <v>0</v>
+      </c>
+      <c r="J14" s="10"/>
+      <c r="K14" s="10" t="s">
         <v>116</v>
       </c>
-      <c r="K14" s="9"/>
       <c r="L14" s="9"/>
       <c r="M14" s="9"/>
       <c r="N14" s="9"/>
@@ -4031,40 +4068,43 @@
       <c r="P14" s="9"/>
       <c r="Q14" s="9"/>
       <c r="R14" s="9"/>
-      <c r="S14" t="str">
+      <c r="S14" s="9"/>
+      <c r="T14" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
+    <row r="15" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>48</v>
+      </c>
+      <c r="B15" t="s">
         <v>126</v>
       </c>
-      <c r="B15" t="s">
-        <v>20</v>
-      </c>
       <c r="C15" t="s">
-        <v>44</v>
-      </c>
-      <c r="D15">
+        <v>20</v>
+      </c>
+      <c r="D15" t="s">
+        <v>44</v>
+      </c>
+      <c r="E15">
         <v>3</v>
       </c>
-      <c r="E15" s="2">
+      <c r="F15" s="2">
         <v>46149.960416666669</v>
       </c>
-      <c r="F15" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="G15">
+      <c r="G15" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="H15">
         <v>114</v>
       </c>
-      <c r="H15">
-        <v>0</v>
-      </c>
-      <c r="J15" t="s">
+      <c r="I15">
+        <v>0</v>
+      </c>
+      <c r="K15" t="s">
         <v>116</v>
       </c>
-      <c r="K15" s="9"/>
       <c r="L15" s="9"/>
       <c r="M15" s="9"/>
       <c r="N15" s="9"/>
@@ -4072,105 +4112,109 @@
       <c r="P15" s="9"/>
       <c r="Q15" s="9"/>
       <c r="R15" s="9"/>
-      <c r="S15" t="str">
+      <c r="S15" s="9"/>
+      <c r="T15" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A16" s="10" t="s">
+    <row r="16" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A16">
+        <v>38</v>
+      </c>
+      <c r="B16" s="10" t="s">
         <v>127</v>
       </c>
-      <c r="B16" s="10" t="s">
+      <c r="C16" s="10" t="s">
         <v>89</v>
       </c>
-      <c r="C16" s="10" t="s">
+      <c r="D16" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="D16" s="10">
-        <v>14</v>
-      </c>
-      <c r="E16" s="11">
+      <c r="E16" s="10">
+        <v>14</v>
+      </c>
+      <c r="F16" s="11">
         <v>46147.338888888888</v>
       </c>
-      <c r="F16" s="10" t="s">
+      <c r="G16" s="10" t="s">
         <v>84</v>
       </c>
-      <c r="G16" s="10">
+      <c r="H16" s="10">
         <v>278</v>
       </c>
-      <c r="H16" s="10">
-        <v>0</v>
-      </c>
-      <c r="I16" s="10" t="s">
+      <c r="I16" s="10">
+        <v>0</v>
+      </c>
+      <c r="J16" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="J16" s="10" t="s">
+      <c r="K16" s="10" t="s">
         <v>116</v>
       </c>
-      <c r="K16" s="9">
+      <c r="L16" s="9">
         <v>5</v>
       </c>
-      <c r="L16" s="9">
+      <c r="M16" s="9">
         <v>3</v>
       </c>
-      <c r="M16" s="9">
-        <v>4</v>
-      </c>
       <c r="N16" s="9">
+        <v>4</v>
+      </c>
+      <c r="O16" s="9">
         <v>5</v>
       </c>
-      <c r="O16" s="9">
-        <v>4</v>
-      </c>
       <c r="P16" s="9">
+        <v>4</v>
+      </c>
+      <c r="Q16" s="9">
         <v>5</v>
-      </c>
-      <c r="Q16" s="9">
-        <v>3</v>
       </c>
       <c r="R16" s="9">
         <v>3</v>
       </c>
-      <c r="S16">
+      <c r="S16" s="9">
+        <v>3</v>
+      </c>
+      <c r="T16">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
     </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
+    <row r="17" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A17">
+        <v>67</v>
+      </c>
+      <c r="B17" t="s">
         <v>129</v>
       </c>
-      <c r="B17" t="s">
+      <c r="C17" t="s">
         <v>89</v>
       </c>
-      <c r="C17" t="s">
+      <c r="D17" t="s">
         <v>18</v>
       </c>
-      <c r="D17">
-        <v>14</v>
-      </c>
-      <c r="E17" s="2">
+      <c r="E17">
+        <v>14</v>
+      </c>
+      <c r="F17" s="2">
         <v>46161.992361111108</v>
       </c>
-      <c r="F17" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="G17">
+      <c r="G17" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="H17">
         <v>5</v>
       </c>
-      <c r="H17">
-        <v>0</v>
-      </c>
-      <c r="J17" t="s">
+      <c r="I17">
+        <v>0</v>
+      </c>
+      <c r="K17" t="s">
         <v>116</v>
       </c>
-      <c r="K17" s="9">
+      <c r="L17" s="9">
         <v>3</v>
       </c>
-      <c r="L17" s="9">
-        <v>4</v>
-      </c>
       <c r="M17" s="9">
         <v>4</v>
       </c>
@@ -4178,120 +4222,126 @@
         <v>4</v>
       </c>
       <c r="O17" s="9">
+        <v>4</v>
+      </c>
+      <c r="P17" s="9">
         <v>3</v>
       </c>
-      <c r="P17" s="9">
-        <v>4</v>
-      </c>
       <c r="Q17" s="9">
+        <v>4</v>
+      </c>
+      <c r="R17" s="9">
         <v>2</v>
       </c>
-      <c r="R17" s="9">
-        <v>4</v>
-      </c>
-      <c r="S17">
+      <c r="S17" s="9">
+        <v>4</v>
+      </c>
+      <c r="T17">
         <f t="shared" si="0"/>
         <v>3.5</v>
       </c>
-      <c r="T17" t="s">
+      <c r="U17" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A18" s="10" t="s">
+    <row r="18" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A18">
+        <v>116</v>
+      </c>
+      <c r="B18" s="10" t="s">
         <v>130</v>
       </c>
-      <c r="B18" s="10" t="s">
+      <c r="C18" s="10" t="s">
         <v>89</v>
       </c>
-      <c r="C18" s="10" t="s">
-        <v>44</v>
-      </c>
-      <c r="D18" s="10">
-        <v>14</v>
-      </c>
-      <c r="E18" s="11">
+      <c r="D18" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="E18" s="10">
+        <v>14</v>
+      </c>
+      <c r="F18" s="11">
         <v>46162.020833333336</v>
       </c>
-      <c r="F18" s="10" t="s">
+      <c r="G18" s="10" t="s">
         <v>84</v>
       </c>
-      <c r="G18" s="10">
+      <c r="H18" s="10">
         <v>15</v>
       </c>
-      <c r="H18" s="10">
-        <v>0</v>
-      </c>
-      <c r="I18" s="10" t="s">
+      <c r="I18" s="10">
+        <v>0</v>
+      </c>
+      <c r="J18" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="J18" s="10" t="s">
+      <c r="K18" s="10" t="s">
         <v>116</v>
       </c>
-      <c r="K18" s="9">
+      <c r="L18" s="9">
         <v>5</v>
       </c>
-      <c r="L18" s="9">
-        <v>4</v>
-      </c>
       <c r="M18" s="9">
         <v>4</v>
       </c>
       <c r="N18" s="9">
+        <v>4</v>
+      </c>
+      <c r="O18" s="9">
         <v>5</v>
       </c>
-      <c r="O18" s="9">
-        <v>4</v>
-      </c>
       <c r="P18" s="9">
+        <v>4</v>
+      </c>
+      <c r="Q18" s="9">
         <v>5</v>
       </c>
-      <c r="Q18" s="9">
-        <v>4</v>
-      </c>
       <c r="R18" s="9">
         <v>4</v>
       </c>
-      <c r="S18">
+      <c r="S18" s="9">
+        <v>4</v>
+      </c>
+      <c r="T18">
         <f t="shared" si="0"/>
         <v>4.375</v>
       </c>
     </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A20" s="10" t="s">
+    <row r="20" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A20">
+        <v>126</v>
+      </c>
+      <c r="B20" s="10" t="s">
         <v>132</v>
       </c>
-      <c r="B20" s="10" t="s">
+      <c r="C20" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="C20" s="10" t="s">
+      <c r="D20" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="D20" s="10">
-        <v>14</v>
-      </c>
-      <c r="E20" s="11">
+      <c r="E20" s="10">
+        <v>14</v>
+      </c>
+      <c r="F20" s="11">
         <v>46175.950694444444</v>
       </c>
-      <c r="F20" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="G20" s="10">
+      <c r="G20" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="H20" s="10">
         <v>1</v>
       </c>
-      <c r="H20" s="10">
-        <v>0</v>
-      </c>
-      <c r="I20" s="10"/>
-      <c r="J20" s="10" t="s">
+      <c r="I20" s="10">
+        <v>0</v>
+      </c>
+      <c r="J20" s="10"/>
+      <c r="K20" s="10" t="s">
         <v>116</v>
       </c>
-      <c r="K20" s="9">
+      <c r="L20" s="9">
         <v>3</v>
       </c>
-      <c r="L20" s="9">
-        <v>4</v>
-      </c>
       <c r="M20" s="9">
         <v>4</v>
       </c>
@@ -4299,59 +4349,62 @@
         <v>4</v>
       </c>
       <c r="O20" s="9">
+        <v>4</v>
+      </c>
+      <c r="P20" s="9">
         <v>2</v>
-      </c>
-      <c r="P20" s="9">
-        <v>3</v>
       </c>
       <c r="Q20" s="9">
         <v>3</v>
       </c>
       <c r="R20" s="9">
-        <v>4</v>
-      </c>
-      <c r="S20">
-        <f t="shared" ref="S20:S28" si="1">IFERROR(AVERAGE(K20:R20),"")</f>
+        <v>3</v>
+      </c>
+      <c r="S20" s="9">
+        <v>4</v>
+      </c>
+      <c r="T20">
+        <f t="shared" ref="T20:T28" si="1">IFERROR(AVERAGE(L20:S20),"")</f>
         <v>3.375</v>
       </c>
-      <c r="T20" t="s">
+      <c r="U20" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="21" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
+    <row r="21" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A21">
+        <v>127</v>
+      </c>
+      <c r="B21" t="s">
         <v>133</v>
       </c>
-      <c r="B21" t="s">
+      <c r="C21" t="s">
         <v>11</v>
       </c>
-      <c r="C21" t="s">
+      <c r="D21" t="s">
         <v>12</v>
       </c>
-      <c r="D21">
-        <v>14</v>
-      </c>
-      <c r="E21" s="2">
+      <c r="E21">
+        <v>14</v>
+      </c>
+      <c r="F21" s="2">
         <v>46175.950694444444</v>
       </c>
-      <c r="F21" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="G21">
+      <c r="G21" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="H21">
         <v>2</v>
       </c>
-      <c r="H21">
-        <v>0</v>
-      </c>
-      <c r="J21" t="s">
+      <c r="I21">
+        <v>0</v>
+      </c>
+      <c r="K21" t="s">
         <v>116</v>
       </c>
-      <c r="K21" s="9">
+      <c r="L21" s="9">
         <v>3</v>
       </c>
-      <c r="L21" s="9">
-        <v>4</v>
-      </c>
       <c r="M21" s="9">
         <v>4</v>
       </c>
@@ -4359,7 +4412,7 @@
         <v>4</v>
       </c>
       <c r="O21" s="9">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P21" s="9">
         <v>3</v>
@@ -4368,48 +4421,51 @@
         <v>3</v>
       </c>
       <c r="R21" s="9">
-        <v>4</v>
-      </c>
-      <c r="S21">
+        <v>3</v>
+      </c>
+      <c r="S21" s="9">
+        <v>4</v>
+      </c>
+      <c r="T21">
         <f t="shared" si="1"/>
         <v>3.5</v>
       </c>
     </row>
-    <row r="22" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A22" s="10" t="s">
+    <row r="22" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A22">
+        <v>86</v>
+      </c>
+      <c r="B22" s="10" t="s">
         <v>134</v>
       </c>
-      <c r="B22" s="10" t="s">
-        <v>20</v>
-      </c>
       <c r="C22" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="D22" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="D22" s="10">
-        <v>14</v>
-      </c>
-      <c r="E22" s="11">
+      <c r="E22" s="10">
+        <v>14</v>
+      </c>
+      <c r="F22" s="11">
         <v>46161.998611111114</v>
       </c>
-      <c r="F22" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="G22" s="10">
+      <c r="G22" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="H22" s="10">
         <v>1</v>
       </c>
-      <c r="H22" s="10">
-        <v>0</v>
-      </c>
-      <c r="I22" s="10"/>
-      <c r="J22" s="10" t="s">
+      <c r="I22" s="10">
+        <v>0</v>
+      </c>
+      <c r="J22" s="10"/>
+      <c r="K22" s="10" t="s">
         <v>116</v>
       </c>
-      <c r="K22" s="9">
+      <c r="L22" s="9">
         <v>2</v>
       </c>
-      <c r="L22" s="9">
-        <v>4</v>
-      </c>
       <c r="M22" s="9">
         <v>4</v>
       </c>
@@ -4417,172 +4473,183 @@
         <v>4</v>
       </c>
       <c r="O22" s="9">
+        <v>4</v>
+      </c>
+      <c r="P22" s="9">
         <v>5</v>
-      </c>
-      <c r="P22" s="9">
-        <v>2</v>
       </c>
       <c r="Q22" s="9">
         <v>2</v>
       </c>
       <c r="R22" s="9">
-        <v>4</v>
-      </c>
-      <c r="S22">
+        <v>2</v>
+      </c>
+      <c r="S22" s="9">
+        <v>4</v>
+      </c>
+      <c r="T22">
         <f t="shared" si="1"/>
         <v>3.375</v>
       </c>
-      <c r="T22" t="s">
+      <c r="U22" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="23" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
+    <row r="23" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A23">
+        <v>87</v>
+      </c>
+      <c r="B23" t="s">
         <v>135</v>
       </c>
-      <c r="B23" t="s">
-        <v>20</v>
-      </c>
       <c r="C23" t="s">
+        <v>20</v>
+      </c>
+      <c r="D23" t="s">
         <v>18</v>
       </c>
-      <c r="D23">
-        <v>14</v>
-      </c>
-      <c r="E23" s="2">
+      <c r="E23">
+        <v>14</v>
+      </c>
+      <c r="F23" s="2">
         <v>46161.998611111114</v>
       </c>
-      <c r="F23" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="G23">
+      <c r="G23" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="H23">
         <v>3</v>
       </c>
-      <c r="H23">
-        <v>0</v>
-      </c>
-      <c r="J23" t="s">
+      <c r="I23">
+        <v>0</v>
+      </c>
+      <c r="K23" t="s">
         <v>116</v>
       </c>
-      <c r="K23" s="9">
-        <v>4</v>
-      </c>
       <c r="L23" s="9">
+        <v>4</v>
+      </c>
+      <c r="M23" s="9">
         <v>3</v>
       </c>
-      <c r="M23" s="9">
-        <v>4</v>
-      </c>
       <c r="N23" s="9">
         <v>4</v>
       </c>
       <c r="O23" s="9">
+        <v>4</v>
+      </c>
+      <c r="P23" s="9">
         <v>3</v>
-      </c>
-      <c r="P23" s="9">
-        <v>2</v>
       </c>
       <c r="Q23" s="9">
         <v>2</v>
       </c>
       <c r="R23" s="9">
-        <v>4</v>
-      </c>
-      <c r="S23">
+        <v>2</v>
+      </c>
+      <c r="S23" s="9">
+        <v>4</v>
+      </c>
+      <c r="T23">
         <f t="shared" si="1"/>
         <v>3.25</v>
       </c>
-      <c r="T23" t="s">
+      <c r="U23" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="24" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A24" s="10" t="s">
+    <row r="24" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A24">
+        <v>75</v>
+      </c>
+      <c r="B24" s="10" t="s">
         <v>136</v>
       </c>
-      <c r="B24" s="10" t="s">
-        <v>20</v>
-      </c>
       <c r="C24" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="D24" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="D24" s="10">
-        <v>14</v>
-      </c>
-      <c r="E24" s="11">
+      <c r="E24" s="10">
+        <v>14</v>
+      </c>
+      <c r="F24" s="11">
         <v>46161.998611111114</v>
       </c>
-      <c r="F24" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="G24" s="10">
+      <c r="G24" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="H24" s="10">
         <v>10</v>
       </c>
-      <c r="H24" s="10">
-        <v>0</v>
-      </c>
-      <c r="I24" s="10"/>
-      <c r="J24" s="10" t="s">
+      <c r="I24" s="10">
+        <v>0</v>
+      </c>
+      <c r="J24" s="10"/>
+      <c r="K24" s="10" t="s">
         <v>116</v>
       </c>
-      <c r="K24" s="9">
-        <v>4</v>
-      </c>
       <c r="L24" s="9">
+        <v>4</v>
+      </c>
+      <c r="M24" s="9">
         <v>3</v>
       </c>
-      <c r="M24" s="9">
-        <v>4</v>
-      </c>
       <c r="N24" s="9">
         <v>4</v>
       </c>
       <c r="O24" s="9">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P24" s="9">
         <v>3</v>
       </c>
       <c r="Q24" s="9">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="R24" s="9">
+        <v>4</v>
+      </c>
+      <c r="S24" s="9">
         <v>3</v>
       </c>
-      <c r="S24">
+      <c r="T24">
         <f t="shared" si="1"/>
         <v>3.5</v>
       </c>
     </row>
-    <row r="25" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
+    <row r="25" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A25">
+        <v>78</v>
+      </c>
+      <c r="B25" t="s">
         <v>137</v>
       </c>
-      <c r="B25" t="s">
-        <v>20</v>
-      </c>
       <c r="C25" t="s">
+        <v>20</v>
+      </c>
+      <c r="D25" t="s">
         <v>18</v>
       </c>
-      <c r="D25">
-        <v>14</v>
-      </c>
-      <c r="E25" s="2">
+      <c r="E25">
+        <v>14</v>
+      </c>
+      <c r="F25" s="2">
         <v>46161.998611111114</v>
       </c>
-      <c r="F25" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="G25">
+      <c r="G25" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="H25">
         <v>2</v>
       </c>
-      <c r="H25">
-        <v>0</v>
-      </c>
-      <c r="J25" t="s">
+      <c r="I25">
+        <v>0</v>
+      </c>
+      <c r="K25" t="s">
         <v>116</v>
       </c>
-      <c r="K25" s="9"/>
       <c r="L25" s="9"/>
       <c r="M25" s="9"/>
       <c r="N25" s="9"/>
@@ -4590,103 +4657,107 @@
       <c r="P25" s="9"/>
       <c r="Q25" s="9"/>
       <c r="R25" s="9"/>
-      <c r="S25" t="str">
+      <c r="S25" s="9"/>
+      <c r="T25" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="26" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A26" s="10" t="s">
+    <row r="26" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A26">
+        <v>84</v>
+      </c>
+      <c r="B26" s="10" t="s">
         <v>138</v>
       </c>
-      <c r="B26" s="10" t="s">
-        <v>20</v>
-      </c>
       <c r="C26" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="D26" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="D26" s="10">
-        <v>14</v>
-      </c>
-      <c r="E26" s="11">
+      <c r="E26" s="10">
+        <v>14</v>
+      </c>
+      <c r="F26" s="11">
         <v>46161.998611111114</v>
       </c>
-      <c r="F26" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="G26" s="10">
+      <c r="G26" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="H26" s="10">
         <v>1</v>
       </c>
-      <c r="H26" s="10">
-        <v>0</v>
-      </c>
-      <c r="I26" s="10"/>
-      <c r="J26" s="10" t="s">
+      <c r="I26" s="10">
+        <v>0</v>
+      </c>
+      <c r="J26" s="10"/>
+      <c r="K26" s="10" t="s">
         <v>116</v>
       </c>
-      <c r="K26" s="9">
+      <c r="L26" s="9">
         <v>3</v>
       </c>
-      <c r="L26" s="9">
+      <c r="M26" s="9">
         <v>5</v>
       </c>
-      <c r="M26" s="9">
-        <v>4</v>
-      </c>
       <c r="N26" s="9">
         <v>4</v>
       </c>
       <c r="O26" s="9">
+        <v>4</v>
+      </c>
+      <c r="P26" s="9">
         <v>5</v>
       </c>
-      <c r="P26" s="9">
+      <c r="Q26" s="9">
         <v>3</v>
       </c>
-      <c r="Q26" s="9">
-        <v>4</v>
-      </c>
       <c r="R26" s="9">
         <v>4</v>
       </c>
-      <c r="S26">
+      <c r="S26" s="9">
+        <v>4</v>
+      </c>
+      <c r="T26">
         <f t="shared" si="1"/>
         <v>4</v>
       </c>
     </row>
-    <row r="27" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A27" t="s">
+    <row r="27" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A27">
+        <v>64</v>
+      </c>
+      <c r="B27" t="s">
         <v>139</v>
       </c>
-      <c r="B27" t="s">
+      <c r="C27" t="s">
         <v>89</v>
       </c>
-      <c r="C27" t="s">
+      <c r="D27" t="s">
         <v>18</v>
       </c>
-      <c r="D27">
-        <v>14</v>
-      </c>
-      <c r="E27" s="2">
+      <c r="E27">
+        <v>14</v>
+      </c>
+      <c r="F27" s="2">
         <v>46161.992361111108</v>
       </c>
-      <c r="F27" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="G27">
+      <c r="G27" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="H27">
         <v>3</v>
       </c>
-      <c r="H27">
-        <v>0</v>
-      </c>
-      <c r="J27" t="s">
+      <c r="I27">
+        <v>0</v>
+      </c>
+      <c r="K27" t="s">
         <v>116</v>
       </c>
-      <c r="K27" s="9">
+      <c r="L27" s="9">
         <v>3</v>
       </c>
-      <c r="L27" s="9">
-        <v>4</v>
-      </c>
       <c r="M27" s="9">
         <v>4</v>
       </c>
@@ -4694,57 +4765,60 @@
         <v>4</v>
       </c>
       <c r="O27" s="9">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P27" s="9">
         <v>3</v>
       </c>
       <c r="Q27" s="9">
+        <v>3</v>
+      </c>
+      <c r="R27" s="9">
         <v>2</v>
       </c>
-      <c r="R27" s="9">
-        <v>4</v>
-      </c>
-      <c r="S27">
+      <c r="S27" s="9">
+        <v>4</v>
+      </c>
+      <c r="T27">
         <f t="shared" si="1"/>
         <v>3.375</v>
       </c>
-      <c r="T27" t="s">
+      <c r="U27" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="28" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A28" s="10" t="s">
+    <row r="28" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A28">
+        <v>71</v>
+      </c>
+      <c r="B28" s="10" t="s">
         <v>140</v>
       </c>
-      <c r="B28" s="10" t="s">
+      <c r="C28" s="10" t="s">
         <v>89</v>
       </c>
-      <c r="C28" s="10" t="s">
+      <c r="D28" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="D28" s="10">
-        <v>14</v>
-      </c>
-      <c r="E28" s="11">
+      <c r="E28" s="10">
+        <v>14</v>
+      </c>
+      <c r="F28" s="11">
         <v>46161.993750000001</v>
       </c>
-      <c r="F28" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="G28" s="10">
+      <c r="G28" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="H28" s="10">
         <v>9</v>
       </c>
-      <c r="H28" s="10">
-        <v>0</v>
-      </c>
-      <c r="I28" s="10"/>
-      <c r="J28" s="10" t="s">
+      <c r="I28" s="10">
+        <v>0</v>
+      </c>
+      <c r="J28" s="10"/>
+      <c r="K28" s="10" t="s">
         <v>116</v>
       </c>
-      <c r="K28" s="9">
-        <v>4</v>
-      </c>
       <c r="L28" s="9">
         <v>4</v>
       </c>
@@ -4755,54 +4829,57 @@
         <v>4</v>
       </c>
       <c r="O28" s="9">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P28" s="9">
         <v>3</v>
       </c>
       <c r="Q28" s="9">
+        <v>3</v>
+      </c>
+      <c r="R28" s="9">
         <v>2</v>
       </c>
-      <c r="R28" s="9">
+      <c r="S28" s="9">
         <v>3</v>
       </c>
-      <c r="S28">
+      <c r="T28">
         <f t="shared" si="1"/>
         <v>3.375</v>
       </c>
-      <c r="T28" t="s">
+      <c r="U28" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="29" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A29" s="14" t="s">
+    <row r="29" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="B29" s="15" t="s">
         <v>131</v>
       </c>
-      <c r="B29" s="14"/>
-      <c r="C29" s="14"/>
-      <c r="D29" s="14"/>
-      <c r="E29" s="14"/>
-      <c r="F29" s="14"/>
-      <c r="G29" s="14"/>
-      <c r="H29" s="14"/>
-      <c r="I29" s="14"/>
-      <c r="J29" s="14"/>
-      <c r="K29" s="14"/>
-      <c r="L29" s="14"/>
-      <c r="M29" s="14"/>
-      <c r="N29" s="14"/>
-      <c r="O29" s="14"/>
-      <c r="P29" s="14"/>
-      <c r="Q29" s="14"/>
-      <c r="R29" s="14"/>
-      <c r="S29" s="14"/>
-      <c r="T29" s="14"/>
+      <c r="C29" s="15"/>
+      <c r="D29" s="15"/>
+      <c r="E29" s="15"/>
+      <c r="F29" s="15"/>
+      <c r="G29" s="15"/>
+      <c r="H29" s="15"/>
+      <c r="I29" s="15"/>
+      <c r="J29" s="15"/>
+      <c r="K29" s="15"/>
+      <c r="L29" s="15"/>
+      <c r="M29" s="15"/>
+      <c r="N29" s="15"/>
+      <c r="O29" s="15"/>
+      <c r="P29" s="15"/>
+      <c r="Q29" s="15"/>
+      <c r="R29" s="15"/>
+      <c r="S29" s="15"/>
+      <c r="T29" s="15"/>
+      <c r="U29" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A1:T1"/>
-    <mergeCell ref="A2:T2"/>
-    <mergeCell ref="A29:T29"/>
+    <mergeCell ref="B1:U1"/>
+    <mergeCell ref="B2:U2"/>
+    <mergeCell ref="B29:U29"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Task 2: add readiness scores for PrintSphere_OLH_en-US_draft02 (avg 3.875)
</commit_message>
<xml_diff>
--- a/doc_readiness_checklist.xlsx
+++ b/doc_readiness_checklist.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\AQCWT\OpenCode_Doc\APAI_Chat\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D6C8872-1C76-4250-947E-B2D01FB77EA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE4B3FF6-0DE1-4E12-9054-4F246F52628A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{BE8B64C7-7DD3-42E9-8432-DA4C4DC91B80}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{BE8B64C7-7DD3-42E9-8432-DA4C4DC91B80}"/>
   </bookViews>
   <sheets>
     <sheet name="All Documents – Status" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="507" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="508" uniqueCount="175">
   <si>
     <t>ID</t>
   </si>
@@ -303,9 +303,6 @@
     <t>Versioning - Basic</t>
   </si>
   <si>
-    <t>PrintSphere_OLH_en-US_draft01</t>
-  </si>
-  <si>
     <t>ProductionCenter_UG_14.0_en-US</t>
   </si>
   <si>
@@ -420,9 +417,6 @@
     <t>Tutorial – Prepress v15: Advanced Job Management</t>
   </si>
   <si>
-    <t>Online Help – PrintSphere: PrintSphere_OLH_en-US_draft01</t>
-  </si>
-  <si>
     <t>User Guide – ProductionCenter: ProductionCenter_UG_14.0_en-US</t>
   </si>
   <si>
@@ -559,6 +553,18 @@
   </si>
   <si>
     <t>★ 116</t>
+  </si>
+  <si>
+    <t>PrintSphere_OLH_en-US_draft02</t>
+  </si>
+  <si>
+    <t>Online Help - PrintSphere: PrintSphere_OLH_en-US_draft02</t>
+  </si>
+  <si>
+    <t>NOT UPLOADED</t>
+  </si>
+  <si>
+    <t>Pending upload — newer version of draft01 (June 2026)</t>
   </si>
 </sst>
 </file>
@@ -694,7 +700,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -711,7 +717,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1095,7 +1100,7 @@
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="B2" t="s">
         <v>10</v>
@@ -1153,7 +1158,7 @@
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B4" t="s">
         <v>15</v>
@@ -1182,7 +1187,7 @@
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="B5" t="s">
         <v>16</v>
@@ -1240,7 +1245,7 @@
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="B7" t="s">
         <v>19</v>
@@ -1298,7 +1303,7 @@
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="B9" t="s">
         <v>22</v>
@@ -1327,7 +1332,7 @@
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="B10" t="s">
         <v>23</v>
@@ -1501,7 +1506,7 @@
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="B16" t="s">
         <v>29</v>
@@ -1530,7 +1535,7 @@
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B17" t="s">
         <v>30</v>
@@ -1588,7 +1593,7 @@
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="B19" t="s">
         <v>32</v>
@@ -1762,7 +1767,7 @@
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="B25" t="s">
         <v>38</v>
@@ -1817,7 +1822,7 @@
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A27" s="4" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="B27" t="s">
         <v>41</v>
@@ -1846,7 +1851,7 @@
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="B28" t="s">
         <v>42</v>
@@ -1904,7 +1909,7 @@
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A30" s="4" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="B30" t="s">
         <v>45</v>
@@ -2165,7 +2170,7 @@
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A39" s="4" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B39" t="s">
         <v>54</v>
@@ -2223,7 +2228,7 @@
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A41" s="4" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="B41" t="s">
         <v>56</v>
@@ -2252,7 +2257,7 @@
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A42" s="4" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="B42" t="s">
         <v>57</v>
@@ -2513,7 +2518,7 @@
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="B51" t="s">
         <v>68</v>
@@ -2803,7 +2808,7 @@
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A61" s="4" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="B61" t="s">
         <v>78</v>
@@ -3009,10 +3014,10 @@
     </row>
     <row r="68" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A68" s="4" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="B68" t="s">
-        <v>87</v>
+        <v>171</v>
       </c>
       <c r="C68" t="s">
         <v>20</v>
@@ -3024,7 +3029,7 @@
         <v>3</v>
       </c>
       <c r="F68" s="2">
-        <v>46149.960416666669</v>
+        <v>46185.443749999999</v>
       </c>
       <c r="G68" s="3" t="s">
         <v>13</v>
@@ -3038,13 +3043,13 @@
     </row>
     <row r="69" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A69" s="4" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="B69" t="s">
+        <v>87</v>
+      </c>
+      <c r="C69" t="s">
         <v>88</v>
-      </c>
-      <c r="C69" t="s">
-        <v>89</v>
       </c>
       <c r="D69" t="s">
         <v>18</v>
@@ -3073,10 +3078,10 @@
         <v>63</v>
       </c>
       <c r="B70" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C70" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D70" t="s">
         <v>18</v>
@@ -3099,13 +3104,13 @@
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="B71" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C71" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D71" t="s">
         <v>18</v>
@@ -3128,13 +3133,13 @@
     </row>
     <row r="72" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="B72" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C72" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D72" t="s">
         <v>18</v>
@@ -3160,10 +3165,10 @@
         <v>66</v>
       </c>
       <c r="B73" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C73" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D73" t="s">
         <v>18</v>
@@ -3186,13 +3191,13 @@
     </row>
     <row r="74" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A74" s="4" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="B74" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C74" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D74" t="s">
         <v>18</v>
@@ -3218,10 +3223,10 @@
         <v>68</v>
       </c>
       <c r="B75" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C75" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D75" t="s">
         <v>18</v>
@@ -3244,13 +3249,13 @@
     </row>
     <row r="76" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A76" s="4" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="B76" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C76" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D76" t="s">
         <v>44</v>
@@ -3279,10 +3284,10 @@
         <v>115</v>
       </c>
       <c r="B77" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C77" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D77" t="s">
         <v>44</v>
@@ -3308,10 +3313,10 @@
         <v>111</v>
       </c>
       <c r="B78" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C78" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D78" t="s">
         <v>44</v>
@@ -3337,10 +3342,10 @@
         <v>112</v>
       </c>
       <c r="B79" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C79" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D79" t="s">
         <v>44</v>
@@ -3366,10 +3371,10 @@
         <v>113</v>
       </c>
       <c r="B80" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C80" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D80" t="s">
         <v>44</v>
@@ -3425,7 +3430,7 @@
   <sheetData>
     <row r="1" spans="1:21" ht="17.399999999999999" x14ac:dyDescent="0.35">
       <c r="B1" s="13" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C1" s="13"/>
       <c r="D1" s="13"/>
@@ -3449,7 +3454,7 @@
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.3">
       <c r="B2" s="14" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C2" s="14"/>
       <c r="D2" s="14"/>
@@ -3472,7 +3477,7 @@
       <c r="U2" s="14"/>
     </row>
     <row r="3" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A3" s="16" t="s">
+      <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B3" s="1" t="s">
@@ -3500,40 +3505,40 @@
         <v>8</v>
       </c>
       <c r="J3" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="K3" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="K3" s="7" t="s">
+      <c r="L3" s="8" t="s">
         <v>104</v>
       </c>
-      <c r="L3" s="8" t="s">
+      <c r="M3" s="8" t="s">
         <v>105</v>
       </c>
-      <c r="M3" s="8" t="s">
+      <c r="N3" s="8" t="s">
         <v>106</v>
       </c>
-      <c r="N3" s="8" t="s">
+      <c r="O3" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="O3" s="8" t="s">
+      <c r="P3" s="8" t="s">
         <v>108</v>
       </c>
-      <c r="P3" s="8" t="s">
+      <c r="Q3" s="8" t="s">
         <v>109</v>
       </c>
-      <c r="Q3" s="8" t="s">
+      <c r="R3" s="8" t="s">
         <v>110</v>
       </c>
-      <c r="R3" s="8" t="s">
+      <c r="S3" s="8" t="s">
         <v>111</v>
       </c>
-      <c r="S3" s="8" t="s">
+      <c r="T3" s="8" t="s">
         <v>112</v>
       </c>
-      <c r="T3" s="8" t="s">
+      <c r="U3" s="8" t="s">
         <v>113</v>
-      </c>
-      <c r="U3" s="8" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="4" spans="1:21" x14ac:dyDescent="0.3">
@@ -3541,7 +3546,7 @@
         <v>124</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C4" s="10" t="s">
         <v>11</v>
@@ -3566,7 +3571,7 @@
       </c>
       <c r="J4" s="10"/>
       <c r="K4" s="10" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="L4" s="9">
         <v>4</v>
@@ -3602,7 +3607,7 @@
         <v>76</v>
       </c>
       <c r="B5" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C5" t="s">
         <v>20</v>
@@ -3626,7 +3631,7 @@
         <v>0</v>
       </c>
       <c r="K5" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="L5" s="9">
         <v>3</v>
@@ -3657,7 +3662,7 @@
         <v>3.5</v>
       </c>
       <c r="U5" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
     </row>
     <row r="6" spans="1:21" x14ac:dyDescent="0.3">
@@ -3665,7 +3670,7 @@
         <v>39</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C6" s="10" t="s">
         <v>20</v>
@@ -3690,7 +3695,7 @@
       </c>
       <c r="J6" s="10"/>
       <c r="K6" s="10" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="L6" s="9"/>
       <c r="M6" s="9"/>
@@ -3710,7 +3715,7 @@
         <v>62</v>
       </c>
       <c r="B7" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C7" t="s">
         <v>20</v>
@@ -3734,7 +3739,7 @@
         <v>0</v>
       </c>
       <c r="K7" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="L7" s="9"/>
       <c r="M7" s="9"/>
@@ -3754,7 +3759,7 @@
         <v>43</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C8" s="10" t="s">
         <v>20</v>
@@ -3779,7 +3784,7 @@
       </c>
       <c r="J8" s="10"/>
       <c r="K8" s="10" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="L8" s="9"/>
       <c r="M8" s="9"/>
@@ -3799,7 +3804,7 @@
         <v>98</v>
       </c>
       <c r="B9" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C9" t="s">
         <v>20</v>
@@ -3823,7 +3828,7 @@
         <v>0</v>
       </c>
       <c r="K9" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="L9" s="9"/>
       <c r="M9" s="9"/>
@@ -3843,7 +3848,7 @@
         <v>95</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C10" s="10" t="s">
         <v>20</v>
@@ -3868,7 +3873,7 @@
       </c>
       <c r="J10" s="10"/>
       <c r="K10" s="10" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="L10" s="9">
         <v>4</v>
@@ -3904,7 +3909,7 @@
         <v>58</v>
       </c>
       <c r="B11" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C11" t="s">
         <v>20</v>
@@ -3929,7 +3934,7 @@
       </c>
       <c r="J11" s="6"/>
       <c r="K11" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="L11" s="9"/>
       <c r="M11" s="9"/>
@@ -3945,7 +3950,7 @@
         <v>45</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C12" s="10" t="s">
         <v>20</v>
@@ -3970,7 +3975,7 @@
       </c>
       <c r="J12" s="10"/>
       <c r="K12" s="10" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="L12" s="9"/>
       <c r="M12" s="9"/>
@@ -3990,7 +3995,7 @@
         <v>44</v>
       </c>
       <c r="B13" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C13" t="s">
         <v>20</v>
@@ -4014,7 +4019,7 @@
         <v>0</v>
       </c>
       <c r="K13" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="L13" s="9"/>
       <c r="M13" s="9"/>
@@ -4034,7 +4039,7 @@
         <v>117</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C14" s="10" t="s">
         <v>20</v>
@@ -4059,7 +4064,7 @@
       </c>
       <c r="J14" s="10"/>
       <c r="K14" s="10" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="L14" s="9"/>
       <c r="M14" s="9"/>
@@ -4075,47 +4080,61 @@
       </c>
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A15">
-        <v>48</v>
-      </c>
       <c r="B15" t="s">
-        <v>126</v>
+        <v>172</v>
       </c>
       <c r="C15" t="s">
         <v>20</v>
       </c>
       <c r="D15" t="s">
-        <v>44</v>
+        <v>18</v>
       </c>
       <c r="E15">
         <v>3</v>
       </c>
-      <c r="F15" s="2">
-        <v>46149.960416666669</v>
-      </c>
+      <c r="F15" s="2"/>
       <c r="G15" s="3" t="s">
-        <v>13</v>
+        <v>173</v>
       </c>
       <c r="H15">
-        <v>114</v>
+        <v>0</v>
       </c>
       <c r="I15">
         <v>0</v>
       </c>
+      <c r="J15" t="s">
+        <v>174</v>
+      </c>
       <c r="K15" t="s">
-        <v>116</v>
-      </c>
-      <c r="L15" s="9"/>
-      <c r="M15" s="9"/>
-      <c r="N15" s="9"/>
-      <c r="O15" s="9"/>
-      <c r="P15" s="9"/>
-      <c r="Q15" s="9"/>
-      <c r="R15" s="9"/>
-      <c r="S15" s="9"/>
-      <c r="T15" t="str">
+        <v>115</v>
+      </c>
+      <c r="L15" s="9">
+        <v>5</v>
+      </c>
+      <c r="M15" s="9">
+        <v>3</v>
+      </c>
+      <c r="N15" s="9">
+        <v>4</v>
+      </c>
+      <c r="O15" s="9">
+        <v>5</v>
+      </c>
+      <c r="P15" s="9">
+        <v>3</v>
+      </c>
+      <c r="Q15" s="9">
+        <v>5</v>
+      </c>
+      <c r="R15" s="9">
+        <v>3</v>
+      </c>
+      <c r="S15" s="9">
+        <v>3</v>
+      </c>
+      <c r="T15">
         <f t="shared" si="0"/>
-        <v/>
+        <v>3.875</v>
       </c>
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.3">
@@ -4123,10 +4142,10 @@
         <v>38</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D16" s="10" t="s">
         <v>18</v>
@@ -4147,10 +4166,10 @@
         <v>0</v>
       </c>
       <c r="J16" s="10" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="K16" s="10" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="L16" s="9">
         <v>5</v>
@@ -4186,10 +4205,10 @@
         <v>67</v>
       </c>
       <c r="B17" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="C17" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D17" t="s">
         <v>18</v>
@@ -4210,7 +4229,7 @@
         <v>0</v>
       </c>
       <c r="K17" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="L17" s="9">
         <v>3</v>
@@ -4241,7 +4260,7 @@
         <v>3.5</v>
       </c>
       <c r="U17" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
     </row>
     <row r="18" spans="1:21" x14ac:dyDescent="0.3">
@@ -4249,10 +4268,10 @@
         <v>116</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D18" s="10" t="s">
         <v>44</v>
@@ -4273,10 +4292,10 @@
         <v>0</v>
       </c>
       <c r="J18" s="10" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="K18" s="10" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="L18" s="9">
         <v>5</v>
@@ -4312,7 +4331,7 @@
         <v>126</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C20" s="10" t="s">
         <v>11</v>
@@ -4337,7 +4356,7 @@
       </c>
       <c r="J20" s="10"/>
       <c r="K20" s="10" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="L20" s="9">
         <v>3</v>
@@ -4368,7 +4387,7 @@
         <v>3.375</v>
       </c>
       <c r="U20" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
     </row>
     <row r="21" spans="1:21" x14ac:dyDescent="0.3">
@@ -4376,7 +4395,7 @@
         <v>127</v>
       </c>
       <c r="B21" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="C21" t="s">
         <v>11</v>
@@ -4400,7 +4419,7 @@
         <v>0</v>
       </c>
       <c r="K21" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="L21" s="9">
         <v>3</v>
@@ -4436,7 +4455,7 @@
         <v>86</v>
       </c>
       <c r="B22" s="10" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="C22" s="10" t="s">
         <v>20</v>
@@ -4461,7 +4480,7 @@
       </c>
       <c r="J22" s="10"/>
       <c r="K22" s="10" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="L22" s="9">
         <v>2</v>
@@ -4492,7 +4511,7 @@
         <v>3.375</v>
       </c>
       <c r="U22" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
     </row>
     <row r="23" spans="1:21" x14ac:dyDescent="0.3">
@@ -4500,7 +4519,7 @@
         <v>87</v>
       </c>
       <c r="B23" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="C23" t="s">
         <v>20</v>
@@ -4524,7 +4543,7 @@
         <v>0</v>
       </c>
       <c r="K23" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="L23" s="9">
         <v>4</v>
@@ -4555,7 +4574,7 @@
         <v>3.25</v>
       </c>
       <c r="U23" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.3">
@@ -4563,7 +4582,7 @@
         <v>75</v>
       </c>
       <c r="B24" s="10" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C24" s="10" t="s">
         <v>20</v>
@@ -4588,7 +4607,7 @@
       </c>
       <c r="J24" s="10"/>
       <c r="K24" s="10" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="L24" s="9">
         <v>4</v>
@@ -4624,7 +4643,7 @@
         <v>78</v>
       </c>
       <c r="B25" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="C25" t="s">
         <v>20</v>
@@ -4648,7 +4667,7 @@
         <v>0</v>
       </c>
       <c r="K25" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="L25" s="9"/>
       <c r="M25" s="9"/>
@@ -4668,7 +4687,7 @@
         <v>84</v>
       </c>
       <c r="B26" s="10" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="C26" s="10" t="s">
         <v>20</v>
@@ -4693,7 +4712,7 @@
       </c>
       <c r="J26" s="10"/>
       <c r="K26" s="10" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="L26" s="9">
         <v>3</v>
@@ -4729,10 +4748,10 @@
         <v>64</v>
       </c>
       <c r="B27" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="C27" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D27" t="s">
         <v>18</v>
@@ -4753,7 +4772,7 @@
         <v>0</v>
       </c>
       <c r="K27" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="L27" s="9">
         <v>3</v>
@@ -4784,7 +4803,7 @@
         <v>3.375</v>
       </c>
       <c r="U27" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="28" spans="1:21" x14ac:dyDescent="0.3">
@@ -4792,10 +4811,10 @@
         <v>71</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D28" s="10" t="s">
         <v>18</v>
@@ -4817,7 +4836,7 @@
       </c>
       <c r="J28" s="10"/>
       <c r="K28" s="10" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="L28" s="9">
         <v>4</v>
@@ -4848,12 +4867,12 @@
         <v>3.375</v>
       </c>
       <c r="U28" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="29" spans="1:21" x14ac:dyDescent="0.3">
       <c r="B29" s="15" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="C29" s="15"/>
       <c r="D29" s="15"/>

</xml_diff>

<commit_message>
Checklist: update draft02 as uploaded (ID=129, COMPLETED, 116 chunks); fix All Documents sheet
</commit_message>
<xml_diff>
--- a/doc_readiness_checklist.xlsx
+++ b/doc_readiness_checklist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\AQCWT\OpenCode_Doc\APAI_Chat\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE4B3FF6-0DE1-4E12-9054-4F246F52628A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{737EB855-22C7-4F2D-ADAD-E4C6DA79CB62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{BE8B64C7-7DD3-42E9-8432-DA4C4DC91B80}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="508" uniqueCount="175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="511" uniqueCount="174">
   <si>
     <t>ID</t>
   </si>
@@ -537,9 +537,6 @@
     <t>★ 117</t>
   </si>
   <si>
-    <t>★ 48</t>
-  </si>
-  <si>
     <t>★ 38</t>
   </si>
   <si>
@@ -561,10 +558,10 @@
     <t>Online Help - PrintSphere: PrintSphere_OLH_en-US_draft02</t>
   </si>
   <si>
-    <t>NOT UPLOADED</t>
-  </si>
-  <si>
-    <t>Pending upload — newer version of draft01 (June 2026)</t>
+    <t>PrintSphere_OLH_en-US_draft01</t>
+  </si>
+  <si>
+    <t>★ 129</t>
   </si>
 </sst>
 </file>
@@ -700,7 +697,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -717,6 +714,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1051,7 +1049,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA2A94EA-D0C4-420F-ADF2-2218BCBD16B2}">
-  <dimension ref="A1:J80"/>
+  <dimension ref="A1:J81"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="6.109375" bestFit="1" customWidth="1"/>
@@ -3013,11 +3011,11 @@
       </c>
     </row>
     <row r="68" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A68" s="4" t="s">
-        <v>165</v>
+      <c r="A68" s="16">
+        <v>48</v>
       </c>
       <c r="B68" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C68" t="s">
         <v>20</v>
@@ -3043,42 +3041,39 @@
     </row>
     <row r="69" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A69" s="4" t="s">
-        <v>166</v>
+        <v>173</v>
       </c>
       <c r="B69" t="s">
-        <v>87</v>
+        <v>170</v>
       </c>
       <c r="C69" t="s">
-        <v>88</v>
+        <v>20</v>
       </c>
       <c r="D69" t="s">
         <v>18</v>
       </c>
       <c r="E69">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="F69" s="2">
-        <v>46147.338888888888</v>
-      </c>
-      <c r="G69" s="6" t="s">
-        <v>84</v>
+        <v>46185.36041666667</v>
+      </c>
+      <c r="G69" s="3" t="s">
+        <v>13</v>
       </c>
       <c r="H69">
-        <v>278</v>
+        <v>116</v>
       </c>
       <c r="I69">
         <v>0</v>
       </c>
-      <c r="J69" s="6" t="s">
-        <v>85</v>
-      </c>
     </row>
     <row r="70" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A70">
-        <v>63</v>
+      <c r="A70" s="4" t="s">
+        <v>165</v>
       </c>
       <c r="B70" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C70" t="s">
         <v>88</v>
@@ -3090,24 +3085,27 @@
         <v>14</v>
       </c>
       <c r="F70" s="2">
-        <v>46161.992361111108</v>
-      </c>
-      <c r="G70" s="3" t="s">
-        <v>13</v>
+        <v>46147.338888888888</v>
+      </c>
+      <c r="G70" s="6" t="s">
+        <v>84</v>
       </c>
       <c r="H70">
-        <v>2</v>
+        <v>278</v>
       </c>
       <c r="I70">
         <v>0</v>
       </c>
+      <c r="J70" s="6" t="s">
+        <v>85</v>
+      </c>
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A71" t="s">
-        <v>167</v>
+      <c r="A71">
+        <v>63</v>
       </c>
       <c r="B71" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C71" t="s">
         <v>88</v>
@@ -3125,7 +3123,7 @@
         <v>13</v>
       </c>
       <c r="H71">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I71">
         <v>0</v>
@@ -3133,10 +3131,10 @@
     </row>
     <row r="72" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="B72" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C72" t="s">
         <v>88</v>
@@ -3148,24 +3146,24 @@
         <v>14</v>
       </c>
       <c r="F72" s="2">
-        <v>46161.993750000001</v>
+        <v>46161.992361111108</v>
       </c>
       <c r="G72" s="3" t="s">
         <v>13</v>
       </c>
       <c r="H72">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="I72">
         <v>0</v>
       </c>
     </row>
     <row r="73" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A73">
-        <v>66</v>
+      <c r="A73" t="s">
+        <v>167</v>
       </c>
       <c r="B73" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C73" t="s">
         <v>88</v>
@@ -3177,24 +3175,24 @@
         <v>14</v>
       </c>
       <c r="F73" s="2">
-        <v>46161.992361111108</v>
+        <v>46161.993750000001</v>
       </c>
       <c r="G73" s="3" t="s">
         <v>13</v>
       </c>
       <c r="H73">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="I73">
         <v>0</v>
       </c>
     </row>
     <row r="74" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A74" s="4" t="s">
-        <v>169</v>
+      <c r="A74">
+        <v>66</v>
       </c>
       <c r="B74" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C74" t="s">
         <v>88</v>
@@ -3212,18 +3210,18 @@
         <v>13</v>
       </c>
       <c r="H74">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I74">
         <v>0</v>
       </c>
     </row>
     <row r="75" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A75">
-        <v>68</v>
+      <c r="A75" s="4" t="s">
+        <v>168</v>
       </c>
       <c r="B75" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C75" t="s">
         <v>88</v>
@@ -3241,50 +3239,47 @@
         <v>13</v>
       </c>
       <c r="H75">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I75">
         <v>0</v>
       </c>
     </row>
     <row r="76" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A76" s="4" t="s">
-        <v>170</v>
+      <c r="A76">
+        <v>68</v>
       </c>
       <c r="B76" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C76" t="s">
         <v>88</v>
       </c>
       <c r="D76" t="s">
-        <v>44</v>
+        <v>18</v>
       </c>
       <c r="E76">
         <v>14</v>
       </c>
       <c r="F76" s="2">
-        <v>46162.020833333336</v>
-      </c>
-      <c r="G76" s="6" t="s">
-        <v>84</v>
+        <v>46161.992361111108</v>
+      </c>
+      <c r="G76" s="3" t="s">
+        <v>13</v>
       </c>
       <c r="H76">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="I76">
         <v>0</v>
       </c>
-      <c r="J76" s="6" t="s">
-        <v>85</v>
-      </c>
     </row>
     <row r="77" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A77">
-        <v>115</v>
+      <c r="A77" s="4" t="s">
+        <v>169</v>
       </c>
       <c r="B77" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C77" t="s">
         <v>88</v>
@@ -3296,24 +3291,27 @@
         <v>14</v>
       </c>
       <c r="F77" s="2">
-        <v>46162.019444444442</v>
-      </c>
-      <c r="G77" s="3" t="s">
-        <v>13</v>
+        <v>46162.020833333336</v>
+      </c>
+      <c r="G77" s="6" t="s">
+        <v>84</v>
       </c>
       <c r="H77">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="I77">
         <v>0</v>
+      </c>
+      <c r="J77" s="6" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="78" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A78">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="B78" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C78" t="s">
         <v>88</v>
@@ -3339,10 +3337,10 @@
     </row>
     <row r="79" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A79">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B79" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C79" t="s">
         <v>88</v>
@@ -3360,7 +3358,7 @@
         <v>13</v>
       </c>
       <c r="H79">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="I79">
         <v>0</v>
@@ -3368,10 +3366,10 @@
     </row>
     <row r="80" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A80">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B80" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C80" t="s">
         <v>88</v>
@@ -3389,9 +3387,38 @@
         <v>13</v>
       </c>
       <c r="H80">
+        <v>10</v>
+      </c>
+      <c r="I80">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A81">
+        <v>113</v>
+      </c>
+      <c r="B81" t="s">
+        <v>99</v>
+      </c>
+      <c r="C81" t="s">
+        <v>88</v>
+      </c>
+      <c r="D81" t="s">
+        <v>44</v>
+      </c>
+      <c r="E81">
+        <v>14</v>
+      </c>
+      <c r="F81" s="2">
+        <v>46162.019444444442</v>
+      </c>
+      <c r="G81" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="H81">
         <v>16</v>
       </c>
-      <c r="I80">
+      <c r="I81">
         <v>0</v>
       </c>
     </row>
@@ -4080,8 +4107,11 @@
       </c>
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>129</v>
+      </c>
       <c r="B15" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C15" t="s">
         <v>20</v>
@@ -4092,18 +4122,17 @@
       <c r="E15">
         <v>3</v>
       </c>
-      <c r="F15" s="2"/>
+      <c r="F15" s="2">
+        <v>46185.36041666667</v>
+      </c>
       <c r="G15" s="3" t="s">
-        <v>173</v>
+        <v>13</v>
       </c>
       <c r="H15">
-        <v>0</v>
+        <v>116</v>
       </c>
       <c r="I15">
         <v>0</v>
-      </c>
-      <c r="J15" t="s">
-        <v>174</v>
       </c>
       <c r="K15" t="s">
         <v>115</v>

</xml_diff>